<commit_message>
XB6A: ngày nghiệm thu bắt đầu 20/8/2026, cột ngày dùng công thức nối tiếp như mẫu XD8 đoạn 1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RHahmApFFRr7mqf4R5YZ3w
</commit_message>
<xml_diff>
--- a/XB6A/1. Danh mục nghiệm thu - XB6A.xlsx
+++ b/XB6A/1. Danh mục nghiệm thu - XB6A.xlsx
@@ -2109,7 +2109,7 @@
       </c>
       <c r="C9" s="18" t="n">
         <f aca="false">'Tuyến XB6A'!C3</f>
-        <v>46248</v>
+        <v>46254</v>
       </c>
       <c r="D9" s="19" t="n">
         <f aca="false">'Tuyến XB6A'!H3</f>
@@ -2139,7 +2139,7 @@
       </c>
       <c r="C10" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C4</f>
-        <v>46249</v>
+        <v>46258</v>
       </c>
       <c r="D10" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H4</f>
@@ -2169,7 +2169,7 @@
       </c>
       <c r="C11" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C5</f>
-        <v>46249</v>
+        <v>46258</v>
       </c>
       <c r="D11" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H5</f>
@@ -2199,7 +2199,7 @@
       </c>
       <c r="C12" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C6</f>
-        <v>46250</v>
+        <v>46259</v>
       </c>
       <c r="D12" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H6</f>
@@ -2229,7 +2229,7 @@
       </c>
       <c r="C13" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C7</f>
-        <v>46251</v>
+        <v>46260</v>
       </c>
       <c r="D13" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H7</f>
@@ -2259,7 +2259,7 @@
       </c>
       <c r="C14" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C8</f>
-        <v>46258</v>
+        <v>46261</v>
       </c>
       <c r="D14" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H8</f>
@@ -2289,7 +2289,7 @@
       </c>
       <c r="C15" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C9</f>
-        <v>46259</v>
+        <v>46262</v>
       </c>
       <c r="D15" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H9</f>
@@ -2319,7 +2319,7 @@
       </c>
       <c r="C16" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C10</f>
-        <v>46260</v>
+        <v>46263</v>
       </c>
       <c r="D16" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H10</f>
@@ -2349,7 +2349,7 @@
       </c>
       <c r="C17" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C11</f>
-        <v>46260</v>
+        <v>46263</v>
       </c>
       <c r="D17" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H11</f>
@@ -2379,7 +2379,7 @@
       </c>
       <c r="C18" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C12</f>
-        <v>46261</v>
+        <v>46264</v>
       </c>
       <c r="D18" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H12</f>
@@ -2409,7 +2409,7 @@
       </c>
       <c r="C19" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C13</f>
-        <v>46261</v>
+        <v>46264</v>
       </c>
       <c r="D19" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H13</f>
@@ -2439,7 +2439,7 @@
       </c>
       <c r="C20" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C14</f>
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="D20" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H14</f>
@@ -2469,7 +2469,7 @@
       </c>
       <c r="C21" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C15</f>
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="D21" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H15</f>
@@ -2499,7 +2499,7 @@
       </c>
       <c r="C22" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C16</f>
-        <v>46263</v>
+        <v>46269</v>
       </c>
       <c r="D22" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H16</f>
@@ -2529,7 +2529,7 @@
       </c>
       <c r="C23" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C17</f>
-        <v>46263</v>
+        <v>46269</v>
       </c>
       <c r="D23" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H17</f>
@@ -2559,7 +2559,7 @@
       </c>
       <c r="C24" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C18</f>
-        <v>46264</v>
+        <v>46270</v>
       </c>
       <c r="D24" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H18</f>
@@ -2589,7 +2589,7 @@
       </c>
       <c r="C25" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C19</f>
-        <v>46268</v>
+        <v>46271</v>
       </c>
       <c r="D25" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H19</f>
@@ -2619,7 +2619,7 @@
       </c>
       <c r="C26" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C20</f>
-        <v>46268</v>
+        <v>46271</v>
       </c>
       <c r="D26" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H20</f>
@@ -2649,7 +2649,7 @@
       </c>
       <c r="C27" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C21</f>
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="D27" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H21</f>
@@ -2679,7 +2679,7 @@
       </c>
       <c r="C28" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C22</f>
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="D28" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H22</f>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="C29" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C23</f>
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="D29" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H23</f>
@@ -2739,7 +2739,7 @@
       </c>
       <c r="C30" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C24</f>
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="D30" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H24</f>
@@ -2769,7 +2769,7 @@
       </c>
       <c r="C31" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C25</f>
-        <v>46271</v>
+        <v>46274</v>
       </c>
       <c r="D31" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H25</f>
@@ -2799,7 +2799,7 @@
       </c>
       <c r="C32" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C26</f>
-        <v>46271</v>
+        <v>46274</v>
       </c>
       <c r="D32" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H26</f>
@@ -2829,7 +2829,7 @@
       </c>
       <c r="C33" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C27</f>
-        <v>46273</v>
+        <v>46276</v>
       </c>
       <c r="D33" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H27</f>
@@ -2859,7 +2859,7 @@
       </c>
       <c r="C34" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C28</f>
-        <v>46275</v>
+        <v>46278</v>
       </c>
       <c r="D34" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H28</f>
@@ -2889,7 +2889,7 @@
       </c>
       <c r="C35" s="29" t="n">
         <f aca="false">'Tuyến XB6A'!C29</f>
-        <v>46277</v>
+        <v>46284</v>
       </c>
       <c r="D35" s="30" t="n">
         <f aca="false">'Tuyến XB6A'!H29</f>
@@ -2919,7 +2919,7 @@
       </c>
       <c r="C36" s="23" t="n">
         <f aca="false">'Tuyến XB6A'!C30</f>
-        <v>46284</v>
+        <v>46286</v>
       </c>
       <c r="D36" s="24" t="n">
         <f aca="false">'Tuyến XB6A'!H30</f>
@@ -3014,7 +3014,7 @@
     <row r="2" s="145" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="144" t="str">
         <f aca="false">"Kèm theo BBNT số: "&amp;VLOOKUP(T2,'Tuyến XB6A'!$A$2:$G$31,7,0)&amp;VLOOKUP(T2,'Tuyến XB6A'!$A$2:$G$31,4,0)</f>
-        <v>Kèm theo BBNT số: 27.NĐXB6A/CVXD ngày 12 tháng 09 năm 2026</v>
+        <v>Kèm theo BBNT số: 27.NĐXB6A/CVXD ngày 19 tháng 09 năm 2026</v>
       </c>
       <c r="B2" s="144"/>
       <c r="C2" s="144"/>
@@ -6749,11 +6749,11 @@
       </c>
       <c r="E22" s="67" t="n">
         <f aca="false">+D22+F22</f>
-        <v>3.733</v>
+        <v>3.763</v>
       </c>
       <c r="F22" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>-0.017</v>
+        <v>0.013</v>
       </c>
       <c r="G22" s="67" t="n">
         <f aca="false">+J22-3.45*2%-(D22-3.45)*6%</f>
@@ -6761,22 +6761,22 @@
       </c>
       <c r="H22" s="67" t="n">
         <f aca="false">G22+I22</f>
-        <v>2.781</v>
+        <v>2.757</v>
       </c>
       <c r="I22" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,70)/1000</f>
-        <v>0.049</v>
+        <v>0.025</v>
       </c>
       <c r="J22" s="67" t="n">
         <v>2.819</v>
       </c>
       <c r="K22" s="67" t="n">
         <f aca="false">J22+L22</f>
-        <v>2.848</v>
+        <v>2.814</v>
       </c>
       <c r="L22" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,70)/1000</f>
-        <v>0.029</v>
+        <v>-0.005</v>
       </c>
       <c r="M22" s="67" t="n">
         <f aca="false">D22</f>
@@ -6784,11 +6784,11 @@
       </c>
       <c r="N22" s="67" t="n">
         <f aca="false">+M22+O22</f>
-        <v>3.735</v>
+        <v>3.731</v>
       </c>
       <c r="O22" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>-0.015</v>
+        <v>-0.019</v>
       </c>
       <c r="P22" s="67" t="n">
         <f aca="false">+J22-3.45*2%-(M22-3.45)*6%</f>
@@ -6796,11 +6796,11 @@
       </c>
       <c r="Q22" s="67" t="n">
         <f aca="false">P22+R22</f>
-        <v>2.724</v>
+        <v>2.745</v>
       </c>
       <c r="R22" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>-0.008</v>
+        <v>0.013</v>
       </c>
       <c r="S22" s="85"/>
       <c r="T22" s="136"/>
@@ -6825,11 +6825,11 @@
       </c>
       <c r="E23" s="67" t="n">
         <f aca="false">+D23+F23</f>
-        <v>3.739</v>
+        <v>3.73</v>
       </c>
       <c r="F23" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>-0.011</v>
+        <v>-0.02</v>
       </c>
       <c r="G23" s="67" t="n">
         <f aca="false">+J23-3.45*2%-(D23-3.45)*6%</f>
@@ -6837,22 +6837,22 @@
       </c>
       <c r="H23" s="67" t="n">
         <f aca="false">G23+I23</f>
-        <v>2.796</v>
+        <v>2.754</v>
       </c>
       <c r="I23" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,70)/1000</f>
-        <v>0.064</v>
+        <v>0.022</v>
       </c>
       <c r="J23" s="67" t="n">
         <v>2.819</v>
       </c>
       <c r="K23" s="67" t="n">
         <f aca="false">J23+L23</f>
-        <v>2.836</v>
+        <v>2.866</v>
       </c>
       <c r="L23" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,70)/1000</f>
-        <v>0.017</v>
+        <v>0.047</v>
       </c>
       <c r="M23" s="67" t="n">
         <f aca="false">D23</f>
@@ -6860,11 +6860,11 @@
       </c>
       <c r="N23" s="67" t="n">
         <f aca="false">+M23+O23</f>
-        <v>3.747</v>
+        <v>3.75</v>
       </c>
       <c r="O23" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>-0.003</v>
+        <v>0</v>
       </c>
       <c r="P23" s="67" t="n">
         <f aca="false">+J23-3.45*2%-(M23-3.45)*6%</f>
@@ -6872,11 +6872,11 @@
       </c>
       <c r="Q23" s="67" t="n">
         <f aca="false">P23+R23</f>
-        <v>2.731</v>
+        <v>2.744</v>
       </c>
       <c r="R23" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>-0.001</v>
+        <v>0.012</v>
       </c>
       <c r="S23" s="85"/>
       <c r="T23" s="136"/>
@@ -6901,11 +6901,11 @@
       </c>
       <c r="E24" s="67" t="n">
         <f aca="false">+D24+F24</f>
-        <v>3.761</v>
+        <v>3.758</v>
       </c>
       <c r="F24" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>0.011</v>
+        <v>0.008</v>
       </c>
       <c r="G24" s="67" t="n">
         <f aca="false">+J24-3.45*2%-(D24-3.45)*6%</f>
@@ -6913,22 +6913,22 @@
       </c>
       <c r="H24" s="67" t="n">
         <f aca="false">G24+I24</f>
-        <v>2.74</v>
+        <v>2.715</v>
       </c>
       <c r="I24" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,70)/1000</f>
-        <v>0.001</v>
+        <v>-0.024</v>
       </c>
       <c r="J24" s="67" t="n">
         <v>2.826</v>
       </c>
       <c r="K24" s="67" t="n">
         <f aca="false">J24+L24</f>
-        <v>2.887</v>
+        <v>2.822</v>
       </c>
       <c r="L24" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,70)/1000</f>
-        <v>0.061</v>
+        <v>-0.004</v>
       </c>
       <c r="M24" s="67" t="n">
         <f aca="false">D24</f>
@@ -6936,11 +6936,11 @@
       </c>
       <c r="N24" s="67" t="n">
         <f aca="false">+M24+O24</f>
-        <v>3.749</v>
+        <v>3.732</v>
       </c>
       <c r="O24" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>-0.001</v>
+        <v>-0.018</v>
       </c>
       <c r="P24" s="67" t="n">
         <f aca="false">+J24-3.45*2%-(M24-3.45)*6%</f>
@@ -6948,11 +6948,11 @@
       </c>
       <c r="Q24" s="67" t="n">
         <f aca="false">P24+R24</f>
-        <v>2.753</v>
+        <v>2.739</v>
       </c>
       <c r="R24" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>0.014</v>
+        <v>0</v>
       </c>
       <c r="S24" s="85"/>
       <c r="T24" s="136"/>
@@ -6989,22 +6989,22 @@
       </c>
       <c r="H25" s="67" t="n">
         <f aca="false">G25+I25</f>
-        <v>2.796</v>
+        <v>2.815</v>
       </c>
       <c r="I25" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,70)/1000</f>
-        <v>0.049</v>
+        <v>0.068</v>
       </c>
       <c r="J25" s="67" t="n">
         <v>2.834</v>
       </c>
       <c r="K25" s="67" t="n">
         <f aca="false">J25+L25</f>
-        <v>2.852</v>
+        <v>2.871</v>
       </c>
       <c r="L25" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,70)/1000</f>
-        <v>0.018</v>
+        <v>0.037</v>
       </c>
       <c r="M25" s="67" t="n">
         <f aca="false">D25</f>
@@ -7012,11 +7012,11 @@
       </c>
       <c r="N25" s="67" t="n">
         <f aca="false">+M25+O25</f>
-        <v>3.77</v>
+        <v>3.74</v>
       </c>
       <c r="O25" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>0.02</v>
+        <v>-0.01</v>
       </c>
       <c r="P25" s="67" t="n">
         <f aca="false">+J25-3.45*2%-(M25-3.45)*6%</f>
@@ -7024,11 +7024,11 @@
       </c>
       <c r="Q25" s="67" t="n">
         <f aca="false">P25+R25</f>
-        <v>2.746</v>
+        <v>2.732</v>
       </c>
       <c r="R25" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>-0.001</v>
+        <v>-0.015</v>
       </c>
       <c r="S25" s="85"/>
       <c r="T25" s="136"/>
@@ -7053,11 +7053,11 @@
       </c>
       <c r="E26" s="67" t="n">
         <f aca="false">+D26+F26</f>
-        <v>3.743</v>
+        <v>3.735</v>
       </c>
       <c r="F26" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>-0.007</v>
+        <v>-0.015</v>
       </c>
       <c r="G26" s="67" t="n">
         <f aca="false">+J26-3.45*2%-(D26-3.45)*6%</f>
@@ -7065,22 +7065,22 @@
       </c>
       <c r="H26" s="67" t="n">
         <f aca="false">G26+I26</f>
-        <v>2.795</v>
+        <v>2.772</v>
       </c>
       <c r="I26" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,70)/1000</f>
-        <v>0.042</v>
+        <v>0.019</v>
       </c>
       <c r="J26" s="67" t="n">
         <v>2.84</v>
       </c>
       <c r="K26" s="67" t="n">
         <f aca="false">J26+L26</f>
-        <v>2.866</v>
+        <v>2.885</v>
       </c>
       <c r="L26" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,70)/1000</f>
-        <v>0.026</v>
+        <v>0.045</v>
       </c>
       <c r="M26" s="67" t="n">
         <f aca="false">D26</f>
@@ -7088,11 +7088,11 @@
       </c>
       <c r="N26" s="67" t="n">
         <f aca="false">+M26+O26</f>
-        <v>3.735</v>
+        <v>3.753</v>
       </c>
       <c r="O26" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>-0.015</v>
+        <v>0.003</v>
       </c>
       <c r="P26" s="67" t="n">
         <f aca="false">+J26-3.45*2%-(M26-3.45)*6%</f>
@@ -7100,11 +7100,11 @@
       </c>
       <c r="Q26" s="67" t="n">
         <f aca="false">P26+R26</f>
-        <v>2.739</v>
+        <v>2.74</v>
       </c>
       <c r="R26" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>-0.014</v>
+        <v>-0.013</v>
       </c>
       <c r="S26" s="85"/>
       <c r="T26" s="136"/>
@@ -7129,11 +7129,11 @@
       </c>
       <c r="E27" s="67" t="n">
         <f aca="false">+D27+F27</f>
-        <v>3.753</v>
+        <v>3.733</v>
       </c>
       <c r="F27" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>0.003</v>
+        <v>-0.017</v>
       </c>
       <c r="G27" s="67" t="n">
         <f aca="false">+J27-3.45*2%-(D27-3.45)*6%</f>
@@ -7141,22 +7141,22 @@
       </c>
       <c r="H27" s="67" t="n">
         <f aca="false">G27+I27</f>
-        <v>2.786</v>
+        <v>2.734</v>
       </c>
       <c r="I27" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,70)/1000</f>
-        <v>0.028</v>
+        <v>-0.024</v>
       </c>
       <c r="J27" s="67" t="n">
         <v>2.845</v>
       </c>
       <c r="K27" s="67" t="n">
         <f aca="false">J27+L27</f>
-        <v>2.845</v>
+        <v>2.88</v>
       </c>
       <c r="L27" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,70)/1000</f>
-        <v>0</v>
+        <v>0.035</v>
       </c>
       <c r="M27" s="67" t="n">
         <f aca="false">D27</f>
@@ -7164,11 +7164,11 @@
       </c>
       <c r="N27" s="67" t="n">
         <f aca="false">+M27+O27</f>
-        <v>3.765</v>
+        <v>3.764</v>
       </c>
       <c r="O27" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>0.015</v>
+        <v>0.014</v>
       </c>
       <c r="P27" s="67" t="n">
         <f aca="false">+J27-3.45*2%-(M27-3.45)*6%</f>
@@ -7176,11 +7176,11 @@
       </c>
       <c r="Q27" s="67" t="n">
         <f aca="false">P27+R27</f>
-        <v>2.777</v>
+        <v>2.764</v>
       </c>
       <c r="R27" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>0.019</v>
+        <v>0.006</v>
       </c>
       <c r="S27" s="85"/>
       <c r="T27" s="136"/>
@@ -7205,11 +7205,11 @@
       </c>
       <c r="E28" s="67" t="n">
         <f aca="false">+D28+F28</f>
-        <v>3.752</v>
+        <v>3.759</v>
       </c>
       <c r="F28" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>0.002</v>
+        <v>0.009</v>
       </c>
       <c r="G28" s="67" t="n">
         <f aca="false">+J28-3.45*2%-(D28-3.45)*6%</f>
@@ -7217,22 +7217,22 @@
       </c>
       <c r="H28" s="67" t="n">
         <f aca="false">G28+I28</f>
-        <v>2.836</v>
+        <v>2.787</v>
       </c>
       <c r="I28" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,70)/1000</f>
-        <v>0.069</v>
+        <v>0.02</v>
       </c>
       <c r="J28" s="67" t="n">
         <v>2.854</v>
       </c>
       <c r="K28" s="67" t="n">
         <f aca="false">J28+L28</f>
-        <v>2.864</v>
+        <v>2.859</v>
       </c>
       <c r="L28" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,70)/1000</f>
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="M28" s="67" t="n">
         <f aca="false">D28</f>
@@ -7240,11 +7240,11 @@
       </c>
       <c r="N28" s="67" t="n">
         <f aca="false">+M28+O28</f>
-        <v>3.761</v>
+        <v>3.764</v>
       </c>
       <c r="O28" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>0.011</v>
+        <v>0.014</v>
       </c>
       <c r="P28" s="67" t="n">
         <f aca="false">+J28-3.45*2%-(M28-3.45)*6%</f>
@@ -7252,11 +7252,11 @@
       </c>
       <c r="Q28" s="67" t="n">
         <f aca="false">P28+R28</f>
-        <v>2.754</v>
+        <v>2.758</v>
       </c>
       <c r="R28" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>-0.013</v>
+        <v>-0.009</v>
       </c>
       <c r="S28" s="85"/>
       <c r="T28" s="136"/>
@@ -7281,11 +7281,11 @@
       </c>
       <c r="E29" s="67" t="n">
         <f aca="false">+D29+F29</f>
-        <v>3.763</v>
+        <v>3.746</v>
       </c>
       <c r="F29" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>0.013</v>
+        <v>-0.004</v>
       </c>
       <c r="G29" s="67" t="n">
         <f aca="false">+J29-3.45*2%-(D29-3.45)*6%</f>
@@ -7293,22 +7293,22 @@
       </c>
       <c r="H29" s="67" t="n">
         <f aca="false">G29+I29</f>
-        <v>2.813</v>
+        <v>2.777</v>
       </c>
       <c r="I29" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,70)/1000</f>
-        <v>0.037</v>
+        <v>0.001</v>
       </c>
       <c r="J29" s="67" t="n">
         <v>2.863</v>
       </c>
       <c r="K29" s="67" t="n">
         <f aca="false">J29+L29</f>
-        <v>2.91</v>
+        <v>2.866</v>
       </c>
       <c r="L29" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,70)/1000</f>
-        <v>0.047</v>
+        <v>0.003</v>
       </c>
       <c r="M29" s="67" t="n">
         <f aca="false">D29</f>
@@ -7316,11 +7316,11 @@
       </c>
       <c r="N29" s="67" t="n">
         <f aca="false">+M29+O29</f>
-        <v>3.73</v>
+        <v>3.744</v>
       </c>
       <c r="O29" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>-0.02</v>
+        <v>-0.006</v>
       </c>
       <c r="P29" s="67" t="n">
         <f aca="false">+J29-3.45*2%-(M29-3.45)*6%</f>
@@ -7328,11 +7328,11 @@
       </c>
       <c r="Q29" s="67" t="n">
         <f aca="false">P29+R29</f>
-        <v>2.76</v>
+        <v>2.792</v>
       </c>
       <c r="R29" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>-0.016</v>
+        <v>0.016</v>
       </c>
       <c r="S29" s="85"/>
       <c r="T29" s="136"/>
@@ -7357,11 +7357,11 @@
       </c>
       <c r="E30" s="67" t="n">
         <f aca="false">+D30+F30</f>
-        <v>3.753</v>
+        <v>3.75</v>
       </c>
       <c r="F30" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>0.003</v>
+        <v>0</v>
       </c>
       <c r="G30" s="67" t="n">
         <f aca="false">+J30-3.45*2%-(D30-3.45)*6%</f>
@@ -7369,22 +7369,22 @@
       </c>
       <c r="H30" s="67" t="n">
         <f aca="false">G30+I30</f>
-        <v>2.812</v>
+        <v>2.776</v>
       </c>
       <c r="I30" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,70)/1000</f>
-        <v>0.036</v>
+        <v>0</v>
       </c>
       <c r="J30" s="67" t="n">
         <v>2.863</v>
       </c>
       <c r="K30" s="67" t="n">
         <f aca="false">J30+L30</f>
-        <v>2.895</v>
+        <v>2.88</v>
       </c>
       <c r="L30" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,70)/1000</f>
-        <v>0.032</v>
+        <v>0.017</v>
       </c>
       <c r="M30" s="67" t="n">
         <f aca="false">D30</f>
@@ -7392,11 +7392,11 @@
       </c>
       <c r="N30" s="67" t="n">
         <f aca="false">+M30+O30</f>
-        <v>3.765</v>
+        <v>3.74</v>
       </c>
       <c r="O30" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>0.015</v>
+        <v>-0.01</v>
       </c>
       <c r="P30" s="67" t="n">
         <f aca="false">+J30-3.45*2%-(M30-3.45)*6%</f>
@@ -7404,11 +7404,11 @@
       </c>
       <c r="Q30" s="67" t="n">
         <f aca="false">P30+R30</f>
-        <v>2.778</v>
+        <v>2.783</v>
       </c>
       <c r="R30" s="67" t="n">
         <f aca="false">RANDBETWEEN(-20,20)/1000</f>
-        <v>0.002</v>
+        <v>0.007</v>
       </c>
       <c r="S30" s="85"/>
       <c r="T30" s="136"/>
@@ -7751,7 +7751,7 @@
     <row r="2" s="145" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="144" t="str">
         <f aca="false">"Kèm theo BBNT số: "&amp;VLOOKUP(L2,'Tuyến XB6A'!$A$2:$G$31,7,0)&amp;VLOOKUP(L2,'Tuyến XB6A'!$A$2:$G$31,4,0)</f>
-        <v>Kèm theo BBNT số: 28.NĐXB6A/CVXD ngày 19 tháng 09 năm 2026</v>
+        <v>Kèm theo BBNT số: 28.NĐXB6A/CVXD ngày 21 tháng 09 năm 2026</v>
       </c>
       <c r="B2" s="144"/>
       <c r="C2" s="144"/>
@@ -8942,11 +8942,11 @@
       </c>
       <c r="F11" s="134" t="n">
         <f aca="false">+E11+G11</f>
-        <v>7.474</v>
+        <v>7.527</v>
       </c>
       <c r="G11" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,110)/1000</f>
-        <v>-0.026</v>
+        <v>0.027</v>
       </c>
       <c r="H11" s="109" t="n">
         <f aca="false">+(E11+E12)/2*D11</f>
@@ -8954,11 +8954,11 @@
       </c>
       <c r="I11" s="109" t="n">
         <f aca="false">+(F11+F12)/2*D11</f>
-        <v>146.79314</v>
+        <v>147.83353</v>
       </c>
       <c r="J11" s="109" t="n">
         <f aca="false">+I11-H11</f>
-        <v>-0.43186</v>
+        <v>0.608530000000002</v>
       </c>
       <c r="K11" s="110"/>
       <c r="M11" s="111"/>
@@ -8984,11 +8984,11 @@
       </c>
       <c r="F12" s="134" t="n">
         <f aca="false">+E12+G12</f>
-        <v>7.482</v>
+        <v>7.535</v>
       </c>
       <c r="G12" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,110)/1000</f>
-        <v>-0.018</v>
+        <v>0.035</v>
       </c>
       <c r="H12" s="109" t="n">
         <f aca="false">+(E12+E13)/2*D12</f>
@@ -8996,11 +8996,11 @@
       </c>
       <c r="I12" s="109" t="n">
         <f aca="false">+(F12+F13)/2*D12</f>
-        <v>129.54765</v>
+        <v>129.693595</v>
       </c>
       <c r="J12" s="109" t="n">
         <f aca="false">+I12-H12</f>
-        <v>0.772649999999999</v>
+        <v>0.918595000000011</v>
       </c>
       <c r="K12" s="110"/>
       <c r="M12" s="111"/>
@@ -9026,11 +9026,11 @@
       </c>
       <c r="F13" s="134" t="n">
         <f aca="false">+E13+G13</f>
-        <v>7.608</v>
+        <v>7.572</v>
       </c>
       <c r="G13" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,110)/1000</f>
-        <v>0.108</v>
+        <v>0.072</v>
       </c>
       <c r="H13" s="109" t="n">
         <f aca="false">+(E13+E14)/2*D13</f>
@@ -9038,11 +9038,11 @@
       </c>
       <c r="I13" s="109" t="n">
         <f aca="false">+(F13+F14)/2*D13</f>
-        <v>130.0526</v>
+        <v>129.97529</v>
       </c>
       <c r="J13" s="109" t="n">
         <f aca="false">+I13-H13</f>
-        <v>1.20260000000002</v>
+        <v>1.12529000000001</v>
       </c>
       <c r="K13" s="110"/>
       <c r="M13" s="111"/>
@@ -9068,11 +9068,11 @@
       </c>
       <c r="F14" s="134" t="n">
         <f aca="false">+E14+G14</f>
-        <v>7.532</v>
+        <v>7.559</v>
       </c>
       <c r="G14" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,110)/1000</f>
-        <v>0.032</v>
+        <v>0.059</v>
       </c>
       <c r="H14" s="109" t="n">
         <f aca="false">+(E14+E15)/2*D14</f>
@@ -9080,11 +9080,11 @@
       </c>
       <c r="I14" s="109" t="n">
         <f aca="false">+(F14+F15)/2*D14</f>
-        <v>97.46955</v>
+        <v>97.98835</v>
       </c>
       <c r="J14" s="109" t="n">
         <f aca="false">+I14-H14</f>
-        <v>0.194550000000007</v>
+        <v>0.713349999999991</v>
       </c>
       <c r="K14" s="110"/>
       <c r="M14" s="111"/>
@@ -9110,11 +9110,11 @@
       </c>
       <c r="F15" s="134" t="n">
         <f aca="false">+E15+G15</f>
-        <v>7.498</v>
+        <v>7.551</v>
       </c>
       <c r="G15" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,110)/1000</f>
-        <v>-0.002</v>
+        <v>0.051</v>
       </c>
       <c r="H15" s="109" t="n">
         <f aca="false">+(E15+E16)/2*D15</f>
@@ -9122,11 +9122,11 @@
       </c>
       <c r="I15" s="109" t="n">
         <f aca="false">+(F15+F16)/2*D15</f>
-        <v>80.62866</v>
+        <v>80.90634</v>
       </c>
       <c r="J15" s="109" t="n">
         <f aca="false">+I15-H15</f>
-        <v>0.528660000000002</v>
+        <v>0.806340000000006</v>
       </c>
       <c r="K15" s="110"/>
       <c r="M15" s="111"/>
@@ -9152,11 +9152,11 @@
       </c>
       <c r="F16" s="134" t="n">
         <f aca="false">+E16+G16</f>
-        <v>7.601</v>
+        <v>7.6</v>
       </c>
       <c r="G16" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,110)/1000</f>
-        <v>0.101</v>
+        <v>0.1</v>
       </c>
       <c r="H16" s="109" t="n">
         <f aca="false">+(E16+E17)/2*D16</f>
@@ -9164,11 +9164,11 @@
       </c>
       <c r="I16" s="109" t="n">
         <f aca="false">+(F16+F17)/2*D16</f>
-        <v>129.676425</v>
+        <v>129.693595</v>
       </c>
       <c r="J16" s="109" t="n">
         <f aca="false">+I16-H16</f>
-        <v>0.901425000000018</v>
+        <v>0.918595000000011</v>
       </c>
       <c r="K16" s="110"/>
       <c r="M16" s="111"/>
@@ -9194,11 +9194,11 @@
       </c>
       <c r="F17" s="134" t="n">
         <f aca="false">+E17+G17</f>
-        <v>7.504</v>
+        <v>7.507</v>
       </c>
       <c r="G17" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,110)/1000</f>
-        <v>0.004</v>
+        <v>0.007</v>
       </c>
       <c r="H17" s="109" t="n">
         <f aca="false">+(E17+E18)/2*D17</f>
@@ -9206,11 +9206,11 @@
       </c>
       <c r="I17" s="109" t="n">
         <f aca="false">+(F17+F18)/2*D17</f>
-        <v>128.886605</v>
+        <v>128.9467</v>
       </c>
       <c r="J17" s="109" t="n">
         <f aca="false">+I17-H17</f>
-        <v>0.111604999999997</v>
+        <v>0.171700000000016</v>
       </c>
       <c r="K17" s="110"/>
       <c r="M17" s="111"/>
@@ -9236,11 +9236,11 @@
       </c>
       <c r="F18" s="134" t="n">
         <f aca="false">+E18+G18</f>
-        <v>7.509</v>
+        <v>7.513</v>
       </c>
       <c r="G18" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,110)/1000</f>
-        <v>0.009</v>
+        <v>0.013</v>
       </c>
       <c r="H18" s="109" t="n">
         <f aca="false">+(E18+E19)/2*D18</f>
@@ -9248,11 +9248,11 @@
       </c>
       <c r="I18" s="109" t="n">
         <f aca="false">+(F18+F19)/2*D18</f>
-        <v>109.493685</v>
+        <v>108.63153</v>
       </c>
       <c r="J18" s="109" t="n">
         <f aca="false">+I18-H18</f>
-        <v>0.818685000000002</v>
+        <v>-0.0434699999999992</v>
       </c>
       <c r="K18" s="110"/>
       <c r="M18" s="111"/>
@@ -9275,11 +9275,11 @@
       </c>
       <c r="F19" s="134" t="n">
         <f aca="false">+E19+G19</f>
-        <v>7.604</v>
+        <v>7.481</v>
       </c>
       <c r="G19" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,110)/1000</f>
-        <v>0.104</v>
+        <v>-0.019</v>
       </c>
       <c r="H19" s="109"/>
       <c r="I19" s="109"/>
@@ -9303,11 +9303,11 @@
       </c>
       <c r="I20" s="150" t="n">
         <f aca="false">SUM(I11:I19)</f>
-        <v>952.548315</v>
+        <v>953.66893</v>
       </c>
       <c r="J20" s="114" t="n">
         <f aca="false">+I20-H20</f>
-        <v>4.09831500000018</v>
+        <v>5.21893000000011</v>
       </c>
       <c r="K20" s="115"/>
       <c r="M20" s="117"/>
@@ -11196,11 +11196,11 @@
         <v>26</v>
       </c>
       <c r="C3" s="44" t="n">
-        <v>46248</v>
+        <v>46254</v>
       </c>
       <c r="D3" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C3,"dd")," tháng ",TEXT(C3,"mm")," năm ",TEXT(C3,"yyyy"))</f>
-        <v>ngày 14 tháng 08 năm 2026</v>
+        <v>ngày 20 tháng 08 năm 2026</v>
       </c>
       <c r="E3" s="38" t="s">
         <v>27</v>
@@ -11229,7 +11229,7 @@
       </c>
       <c r="M3" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C3,"dd"))</f>
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="N3" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C3,"mm"))</f>
@@ -11257,11 +11257,12 @@
         <v>31</v>
       </c>
       <c r="C4" s="44" t="n">
-        <v>46249</v>
+        <f aca="false">+C3+4</f>
+        <v>46258</v>
       </c>
       <c r="D4" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C4,"dd")," tháng ",TEXT(C4,"mm")," năm ",TEXT(C4,"yyyy"))</f>
-        <v>ngày 15 tháng 08 năm 2026</v>
+        <v>ngày 24 tháng 08 năm 2026</v>
       </c>
       <c r="E4" s="38" t="s">
         <v>27</v>
@@ -11292,7 +11293,7 @@
       </c>
       <c r="M4" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C4,"dd"))</f>
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="N4" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C4,"mm"))</f>
@@ -11320,11 +11321,12 @@
         <v>33</v>
       </c>
       <c r="C5" s="44" t="n">
-        <v>46249</v>
+        <f aca="false">+C4</f>
+        <v>46258</v>
       </c>
       <c r="D5" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C5,"dd")," tháng ",TEXT(C5,"mm")," năm ",TEXT(C5,"yyyy"))</f>
-        <v>ngày 15 tháng 08 năm 2026</v>
+        <v>ngày 24 tháng 08 năm 2026</v>
       </c>
       <c r="E5" s="38" t="s">
         <v>27</v>
@@ -11355,7 +11357,7 @@
       </c>
       <c r="M5" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C5,"dd"))</f>
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="N5" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C5,"mm"))</f>
@@ -11383,11 +11385,12 @@
         <v>35</v>
       </c>
       <c r="C6" s="44" t="n">
-        <v>46250</v>
+        <f aca="false">+C5+1</f>
+        <v>46259</v>
       </c>
       <c r="D6" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C6,"dd")," tháng ",TEXT(C6,"mm")," năm ",TEXT(C6,"yyyy"))</f>
-        <v>ngày 16 tháng 08 năm 2026</v>
+        <v>ngày 25 tháng 08 năm 2026</v>
       </c>
       <c r="E6" s="38" t="s">
         <v>27</v>
@@ -11418,7 +11421,7 @@
       </c>
       <c r="M6" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C6,"dd"))</f>
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="N6" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C6,"mm"))</f>
@@ -11446,11 +11449,12 @@
         <v>36</v>
       </c>
       <c r="C7" s="44" t="n">
-        <v>46251</v>
+        <f aca="false">+C6+1</f>
+        <v>46260</v>
       </c>
       <c r="D7" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C7,"dd")," tháng ",TEXT(C7,"mm")," năm ",TEXT(C7,"yyyy"))</f>
-        <v>ngày 17 tháng 08 năm 2026</v>
+        <v>ngày 26 tháng 08 năm 2026</v>
       </c>
       <c r="E7" s="38" t="s">
         <v>27</v>
@@ -11481,7 +11485,7 @@
       </c>
       <c r="M7" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C7,"dd"))</f>
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="N7" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C7,"mm"))</f>
@@ -11509,11 +11513,12 @@
         <v>37</v>
       </c>
       <c r="C8" s="44" t="n">
-        <v>46258</v>
+        <f aca="false">+C7+1</f>
+        <v>46261</v>
       </c>
       <c r="D8" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C8,"dd")," tháng ",TEXT(C8,"mm")," năm ",TEXT(C8,"yyyy"))</f>
-        <v>ngày 24 tháng 08 năm 2026</v>
+        <v>ngày 27 tháng 08 năm 2026</v>
       </c>
       <c r="E8" s="38" t="s">
         <v>27</v>
@@ -11544,7 +11549,7 @@
       </c>
       <c r="M8" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C8,"dd"))</f>
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="N8" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C8,"mm"))</f>
@@ -11572,11 +11577,12 @@
         <v>38</v>
       </c>
       <c r="C9" s="44" t="n">
-        <v>46259</v>
+        <f aca="false">+C8+1</f>
+        <v>46262</v>
       </c>
       <c r="D9" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C9,"dd")," tháng ",TEXT(C9,"mm")," năm ",TEXT(C9,"yyyy"))</f>
-        <v>ngày 25 tháng 08 năm 2026</v>
+        <v>ngày 28 tháng 08 năm 2026</v>
       </c>
       <c r="E9" s="38" t="s">
         <v>27</v>
@@ -11607,7 +11613,7 @@
       </c>
       <c r="M9" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C9,"dd"))</f>
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N9" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C9,"mm"))</f>
@@ -11635,11 +11641,12 @@
         <v>39</v>
       </c>
       <c r="C10" s="44" t="n">
-        <v>46260</v>
+        <f aca="false">+C9+1</f>
+        <v>46263</v>
       </c>
       <c r="D10" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C10,"dd")," tháng ",TEXT(C10,"mm")," năm ",TEXT(C10,"yyyy"))</f>
-        <v>ngày 26 tháng 08 năm 2026</v>
+        <v>ngày 29 tháng 08 năm 2026</v>
       </c>
       <c r="E10" s="38" t="s">
         <v>27</v>
@@ -11670,7 +11677,7 @@
       </c>
       <c r="M10" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C10,"dd"))</f>
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="N10" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C10,"mm"))</f>
@@ -11698,11 +11705,12 @@
         <v>40</v>
       </c>
       <c r="C11" s="44" t="n">
-        <v>46260</v>
+        <f aca="false">+C10</f>
+        <v>46263</v>
       </c>
       <c r="D11" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C11,"dd")," tháng ",TEXT(C11,"mm")," năm ",TEXT(C11,"yyyy"))</f>
-        <v>ngày 26 tháng 08 năm 2026</v>
+        <v>ngày 29 tháng 08 năm 2026</v>
       </c>
       <c r="E11" s="38" t="s">
         <v>27</v>
@@ -11733,7 +11741,7 @@
       </c>
       <c r="M11" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C11,"dd"))</f>
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="N11" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C11,"mm"))</f>
@@ -11761,11 +11769,12 @@
         <v>41</v>
       </c>
       <c r="C12" s="44" t="n">
-        <v>46261</v>
+        <f aca="false">+C11+1</f>
+        <v>46264</v>
       </c>
       <c r="D12" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C12,"dd")," tháng ",TEXT(C12,"mm")," năm ",TEXT(C12,"yyyy"))</f>
-        <v>ngày 27 tháng 08 năm 2026</v>
+        <v>ngày 30 tháng 08 năm 2026</v>
       </c>
       <c r="E12" s="38" t="s">
         <v>27</v>
@@ -11796,7 +11805,7 @@
       </c>
       <c r="M12" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C12,"dd"))</f>
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="N12" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C12,"mm"))</f>
@@ -11824,11 +11833,12 @@
         <v>42</v>
       </c>
       <c r="C13" s="44" t="n">
-        <v>46261</v>
+        <f aca="false">+C12</f>
+        <v>46264</v>
       </c>
       <c r="D13" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C13,"dd")," tháng ",TEXT(C13,"mm")," năm ",TEXT(C13,"yyyy"))</f>
-        <v>ngày 27 tháng 08 năm 2026</v>
+        <v>ngày 30 tháng 08 năm 2026</v>
       </c>
       <c r="E13" s="38" t="s">
         <v>27</v>
@@ -11859,7 +11869,7 @@
       </c>
       <c r="M13" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C13,"dd"))</f>
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="N13" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C13,"mm"))</f>
@@ -11887,11 +11897,12 @@
         <v>43</v>
       </c>
       <c r="C14" s="44" t="n">
-        <v>46262</v>
+        <f aca="false">+C13+4</f>
+        <v>46268</v>
       </c>
       <c r="D14" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C14,"dd")," tháng ",TEXT(C14,"mm")," năm ",TEXT(C14,"yyyy"))</f>
-        <v>ngày 28 tháng 08 năm 2026</v>
+        <v>ngày 03 tháng 09 năm 2026</v>
       </c>
       <c r="E14" s="38" t="s">
         <v>27</v>
@@ -11922,11 +11933,11 @@
       </c>
       <c r="M14" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C14,"dd"))</f>
-        <v>28</v>
+        <v>03</v>
       </c>
       <c r="N14" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C14,"mm"))</f>
-        <v>08</v>
+        <v>09</v>
       </c>
       <c r="O14" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C14,"yyyy"))</f>
@@ -11950,11 +11961,12 @@
         <v>44</v>
       </c>
       <c r="C15" s="44" t="n">
-        <v>46262</v>
+        <f aca="false">+C14</f>
+        <v>46268</v>
       </c>
       <c r="D15" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C15,"dd")," tháng ",TEXT(C15,"mm")," năm ",TEXT(C15,"yyyy"))</f>
-        <v>ngày 28 tháng 08 năm 2026</v>
+        <v>ngày 03 tháng 09 năm 2026</v>
       </c>
       <c r="E15" s="38" t="s">
         <v>27</v>
@@ -11985,11 +11997,11 @@
       </c>
       <c r="M15" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C15,"dd"))</f>
-        <v>28</v>
+        <v>03</v>
       </c>
       <c r="N15" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C15,"mm"))</f>
-        <v>08</v>
+        <v>09</v>
       </c>
       <c r="O15" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C15,"yyyy"))</f>
@@ -12013,11 +12025,12 @@
         <v>45</v>
       </c>
       <c r="C16" s="44" t="n">
-        <v>46263</v>
+        <f aca="false">+C15+1</f>
+        <v>46269</v>
       </c>
       <c r="D16" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C16,"dd")," tháng ",TEXT(C16,"mm")," năm ",TEXT(C16,"yyyy"))</f>
-        <v>ngày 29 tháng 08 năm 2026</v>
+        <v>ngày 04 tháng 09 năm 2026</v>
       </c>
       <c r="E16" s="38" t="s">
         <v>27</v>
@@ -12048,11 +12061,11 @@
       </c>
       <c r="M16" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C16,"dd"))</f>
-        <v>29</v>
+        <v>04</v>
       </c>
       <c r="N16" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C16,"mm"))</f>
-        <v>08</v>
+        <v>09</v>
       </c>
       <c r="O16" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C16,"yyyy"))</f>
@@ -12076,11 +12089,12 @@
         <v>46</v>
       </c>
       <c r="C17" s="44" t="n">
-        <v>46263</v>
+        <f aca="false">+C16</f>
+        <v>46269</v>
       </c>
       <c r="D17" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C17,"dd")," tháng ",TEXT(C17,"mm")," năm ",TEXT(C17,"yyyy"))</f>
-        <v>ngày 29 tháng 08 năm 2026</v>
+        <v>ngày 04 tháng 09 năm 2026</v>
       </c>
       <c r="E17" s="38" t="s">
         <v>27</v>
@@ -12111,11 +12125,11 @@
       </c>
       <c r="M17" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C17,"dd"))</f>
-        <v>29</v>
+        <v>04</v>
       </c>
       <c r="N17" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C17,"mm"))</f>
-        <v>08</v>
+        <v>09</v>
       </c>
       <c r="O17" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C17,"yyyy"))</f>
@@ -12139,11 +12153,12 @@
         <v>47</v>
       </c>
       <c r="C18" s="44" t="n">
-        <v>46264</v>
+        <f aca="false">+C17+1</f>
+        <v>46270</v>
       </c>
       <c r="D18" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C18,"dd")," tháng ",TEXT(C18,"mm")," năm ",TEXT(C18,"yyyy"))</f>
-        <v>ngày 30 tháng 08 năm 2026</v>
+        <v>ngày 05 tháng 09 năm 2026</v>
       </c>
       <c r="E18" s="38" t="s">
         <v>27</v>
@@ -12174,11 +12189,11 @@
       </c>
       <c r="M18" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C18,"dd"))</f>
-        <v>30</v>
+        <v>05</v>
       </c>
       <c r="N18" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C18,"mm"))</f>
-        <v>08</v>
+        <v>09</v>
       </c>
       <c r="O18" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C18,"yyyy"))</f>
@@ -12202,11 +12217,12 @@
         <v>48</v>
       </c>
       <c r="C19" s="44" t="n">
-        <v>46268</v>
+        <f aca="false">+C18+1</f>
+        <v>46271</v>
       </c>
       <c r="D19" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C19,"dd")," tháng ",TEXT(C19,"mm")," năm ",TEXT(C19,"yyyy"))</f>
-        <v>ngày 03 tháng 09 năm 2026</v>
+        <v>ngày 06 tháng 09 năm 2026</v>
       </c>
       <c r="E19" s="38" t="s">
         <v>27</v>
@@ -12237,7 +12253,7 @@
       </c>
       <c r="M19" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C19,"dd"))</f>
-        <v>03</v>
+        <v>06</v>
       </c>
       <c r="N19" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C19,"mm"))</f>
@@ -12265,11 +12281,12 @@
         <v>49</v>
       </c>
       <c r="C20" s="44" t="n">
-        <v>46268</v>
+        <f aca="false">+C19</f>
+        <v>46271</v>
       </c>
       <c r="D20" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C20,"dd")," tháng ",TEXT(C20,"mm")," năm ",TEXT(C20,"yyyy"))</f>
-        <v>ngày 03 tháng 09 năm 2026</v>
+        <v>ngày 06 tháng 09 năm 2026</v>
       </c>
       <c r="E20" s="38" t="s">
         <v>27</v>
@@ -12300,7 +12317,7 @@
       </c>
       <c r="M20" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C20,"dd"))</f>
-        <v>03</v>
+        <v>06</v>
       </c>
       <c r="N20" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C20,"mm"))</f>
@@ -12328,11 +12345,12 @@
         <v>50</v>
       </c>
       <c r="C21" s="44" t="n">
-        <v>46269</v>
+        <f aca="false">+C20+1</f>
+        <v>46272</v>
       </c>
       <c r="D21" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C21,"dd")," tháng ",TEXT(C21,"mm")," năm ",TEXT(C21,"yyyy"))</f>
-        <v>ngày 04 tháng 09 năm 2026</v>
+        <v>ngày 07 tháng 09 năm 2026</v>
       </c>
       <c r="E21" s="38" t="s">
         <v>27</v>
@@ -12363,7 +12381,7 @@
       </c>
       <c r="M21" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C21,"dd"))</f>
-        <v>04</v>
+        <v>07</v>
       </c>
       <c r="N21" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C21,"mm"))</f>
@@ -12391,11 +12409,12 @@
         <v>51</v>
       </c>
       <c r="C22" s="44" t="n">
-        <v>46269</v>
+        <f aca="false">+C21</f>
+        <v>46272</v>
       </c>
       <c r="D22" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C22,"dd")," tháng ",TEXT(C22,"mm")," năm ",TEXT(C22,"yyyy"))</f>
-        <v>ngày 04 tháng 09 năm 2026</v>
+        <v>ngày 07 tháng 09 năm 2026</v>
       </c>
       <c r="E22" s="38" t="s">
         <v>27</v>
@@ -12426,7 +12445,7 @@
       </c>
       <c r="M22" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C22,"dd"))</f>
-        <v>04</v>
+        <v>07</v>
       </c>
       <c r="N22" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C22,"mm"))</f>
@@ -12454,11 +12473,12 @@
         <v>52</v>
       </c>
       <c r="C23" s="44" t="n">
-        <v>46270</v>
+        <f aca="false">+C22+1</f>
+        <v>46273</v>
       </c>
       <c r="D23" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C23,"dd")," tháng ",TEXT(C23,"mm")," năm ",TEXT(C23,"yyyy"))</f>
-        <v>ngày 05 tháng 09 năm 2026</v>
+        <v>ngày 08 tháng 09 năm 2026</v>
       </c>
       <c r="E23" s="38" t="s">
         <v>27</v>
@@ -12489,7 +12509,7 @@
       </c>
       <c r="M23" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C23,"dd"))</f>
-        <v>05</v>
+        <v>08</v>
       </c>
       <c r="N23" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C23,"mm"))</f>
@@ -12517,11 +12537,12 @@
         <v>54</v>
       </c>
       <c r="C24" s="44" t="n">
-        <v>46270</v>
+        <f aca="false">+C23</f>
+        <v>46273</v>
       </c>
       <c r="D24" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C24,"dd")," tháng ",TEXT(C24,"mm")," năm ",TEXT(C24,"yyyy"))</f>
-        <v>ngày 05 tháng 09 năm 2026</v>
+        <v>ngày 08 tháng 09 năm 2026</v>
       </c>
       <c r="E24" s="38" t="s">
         <v>27</v>
@@ -12552,7 +12573,7 @@
       </c>
       <c r="M24" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C24,"dd"))</f>
-        <v>05</v>
+        <v>08</v>
       </c>
       <c r="N24" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C24,"mm"))</f>
@@ -12580,11 +12601,12 @@
         <v>55</v>
       </c>
       <c r="C25" s="44" t="n">
-        <v>46271</v>
+        <f aca="false">+C24+1</f>
+        <v>46274</v>
       </c>
       <c r="D25" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C25,"dd")," tháng ",TEXT(C25,"mm")," năm ",TEXT(C25,"yyyy"))</f>
-        <v>ngày 06 tháng 09 năm 2026</v>
+        <v>ngày 09 tháng 09 năm 2026</v>
       </c>
       <c r="E25" s="38" t="s">
         <v>27</v>
@@ -12615,7 +12637,7 @@
       </c>
       <c r="M25" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C25,"dd"))</f>
-        <v>06</v>
+        <v>09</v>
       </c>
       <c r="N25" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C25,"mm"))</f>
@@ -12643,11 +12665,12 @@
         <v>56</v>
       </c>
       <c r="C26" s="44" t="n">
-        <v>46271</v>
+        <f aca="false">+C25</f>
+        <v>46274</v>
       </c>
       <c r="D26" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C26,"dd")," tháng ",TEXT(C26,"mm")," năm ",TEXT(C26,"yyyy"))</f>
-        <v>ngày 06 tháng 09 năm 2026</v>
+        <v>ngày 09 tháng 09 năm 2026</v>
       </c>
       <c r="E26" s="38" t="s">
         <v>27</v>
@@ -12678,7 +12701,7 @@
       </c>
       <c r="M26" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C26,"dd"))</f>
-        <v>06</v>
+        <v>09</v>
       </c>
       <c r="N26" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C26,"mm"))</f>
@@ -12706,11 +12729,12 @@
         <v>57</v>
       </c>
       <c r="C27" s="44" t="n">
-        <v>46273</v>
+        <f aca="false">+C26+2</f>
+        <v>46276</v>
       </c>
       <c r="D27" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C27,"dd")," tháng ",TEXT(C27,"mm")," năm ",TEXT(C27,"yyyy"))</f>
-        <v>ngày 08 tháng 09 năm 2026</v>
+        <v>ngày 11 tháng 09 năm 2026</v>
       </c>
       <c r="E27" s="38" t="s">
         <v>27</v>
@@ -12739,7 +12763,7 @@
       </c>
       <c r="M27" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C27,"dd"))</f>
-        <v>08</v>
+        <v>11</v>
       </c>
       <c r="N27" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C27,"mm"))</f>
@@ -12767,11 +12791,12 @@
         <v>58</v>
       </c>
       <c r="C28" s="44" t="n">
-        <v>46275</v>
+        <f aca="false">+C27+2</f>
+        <v>46278</v>
       </c>
       <c r="D28" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C28,"dd")," tháng ",TEXT(C28,"mm")," năm ",TEXT(C28,"yyyy"))</f>
-        <v>ngày 10 tháng 09 năm 2026</v>
+        <v>ngày 13 tháng 09 năm 2026</v>
       </c>
       <c r="E28" s="38" t="s">
         <v>27</v>
@@ -12802,7 +12827,7 @@
       </c>
       <c r="M28" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C28,"dd"))</f>
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="N28" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C28,"mm"))</f>
@@ -12830,11 +12855,12 @@
         <v>60</v>
       </c>
       <c r="C29" s="44" t="n">
-        <v>46277</v>
+        <f aca="false">+C28+6</f>
+        <v>46284</v>
       </c>
       <c r="D29" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C29,"dd")," tháng ",TEXT(C29,"mm")," năm ",TEXT(C29,"yyyy"))</f>
-        <v>ngày 12 tháng 09 năm 2026</v>
+        <v>ngày 19 tháng 09 năm 2026</v>
       </c>
       <c r="E29" s="38" t="s">
         <v>27</v>
@@ -12865,7 +12891,7 @@
       </c>
       <c r="M29" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C29,"dd"))</f>
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="N29" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C29,"mm"))</f>
@@ -12893,11 +12919,12 @@
         <v>61</v>
       </c>
       <c r="C30" s="44" t="n">
-        <v>46284</v>
+        <f aca="false">+C29+2</f>
+        <v>46286</v>
       </c>
       <c r="D30" s="39" t="str">
         <f aca="false">CONCATENATE("ngày ",TEXT(C30,"dd")," tháng ",TEXT(C30,"mm")," năm ",TEXT(C30,"yyyy"))</f>
-        <v>ngày 19 tháng 09 năm 2026</v>
+        <v>ngày 21 tháng 09 năm 2026</v>
       </c>
       <c r="E30" s="38" t="s">
         <v>27</v>
@@ -12928,7 +12955,7 @@
       </c>
       <c r="M30" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C30,"dd"))</f>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="N30" s="39" t="str">
         <f aca="false">CONCATENATE(TEXT(C30,"mm"))</f>
@@ -13475,7 +13502,7 @@
     <row r="2" s="56" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="54" t="str">
         <f aca="false">"Kèm theo BBNT số: "&amp;VLOOKUP(T2,'Tuyến XB6A'!$A$2:$G$29,7,0)&amp;VLOOKUP(T2,'Tuyến XB6A'!$A$2:$G$29,4,0)</f>
-        <v>Kèm theo BBNT số: 01.NĐXB6A/CVXD ngày 14 tháng 08 năm 2026</v>
+        <v>Kèm theo BBNT số: 01.NĐXB6A/CVXD ngày 20 tháng 08 năm 2026</v>
       </c>
       <c r="B2" s="54"/>
       <c r="C2" s="54"/>
@@ -13766,55 +13793,55 @@
       </c>
       <c r="E12" s="66" t="n">
         <f aca="false">D12+F12</f>
-        <v>0.023</v>
+        <v>-0.02</v>
       </c>
       <c r="F12" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>-0.027</v>
+        <v>-0.07</v>
       </c>
       <c r="G12" s="66" t="n">
         <v>0.07</v>
       </c>
       <c r="H12" s="66" t="n">
         <f aca="false">G12+I12</f>
-        <v>0.086</v>
+        <v>0.031</v>
       </c>
       <c r="I12" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>0.016</v>
+        <v>-0.039</v>
       </c>
       <c r="J12" s="66" t="n">
         <v>0.09</v>
       </c>
       <c r="K12" s="66" t="n">
         <f aca="false">J12+L12</f>
-        <v>0.112</v>
+        <v>0.029</v>
       </c>
       <c r="L12" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>0.022</v>
+        <v>-0.061</v>
       </c>
       <c r="M12" s="66" t="n">
         <v>0.06</v>
       </c>
       <c r="N12" s="66" t="n">
         <f aca="false">M12+O12</f>
-        <v>-0.011</v>
+        <v>-0.005</v>
       </c>
       <c r="O12" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>-0.071</v>
+        <v>-0.065</v>
       </c>
       <c r="P12" s="66" t="n">
         <v>0.02</v>
       </c>
       <c r="Q12" s="66" t="n">
         <f aca="false">P12+R12</f>
-        <v>-0.024</v>
+        <v>0.034</v>
       </c>
       <c r="R12" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>-0.044</v>
+        <v>0.014</v>
       </c>
       <c r="S12" s="66"/>
       <c r="T12" s="52" t="n">
@@ -13837,55 +13864,55 @@
       </c>
       <c r="E13" s="66" t="n">
         <f aca="false">D13+F13</f>
-        <v>0.128</v>
+        <v>0.029</v>
       </c>
       <c r="F13" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>0.088</v>
+        <v>-0.011</v>
       </c>
       <c r="G13" s="66" t="n">
         <v>0.05</v>
       </c>
       <c r="H13" s="66" t="n">
         <f aca="false">G13+I13</f>
-        <v>0.052</v>
+        <v>-0.04</v>
       </c>
       <c r="I13" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>0.002</v>
+        <v>-0.09</v>
       </c>
       <c r="J13" s="66" t="n">
         <v>0.05</v>
       </c>
       <c r="K13" s="66" t="n">
         <f aca="false">J13+L13</f>
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="L13" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>-0.05</v>
+        <v>0.1</v>
       </c>
       <c r="M13" s="66" t="n">
         <v>0.03</v>
       </c>
       <c r="N13" s="66" t="n">
         <f aca="false">M13+O13</f>
-        <v>-0.045</v>
+        <v>0.117</v>
       </c>
       <c r="O13" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>-0.075</v>
+        <v>0.087</v>
       </c>
       <c r="P13" s="66" t="n">
         <v>0.01</v>
       </c>
       <c r="Q13" s="66" t="n">
         <f aca="false">P13+R13</f>
-        <v>0.015</v>
+        <v>0.039</v>
       </c>
       <c r="R13" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>0.005</v>
+        <v>0.029</v>
       </c>
       <c r="S13" s="66"/>
       <c r="T13" s="52" t="n">
@@ -13908,55 +13935,55 @@
       </c>
       <c r="E14" s="66" t="n">
         <f aca="false">D14+F14</f>
-        <v>-0.086</v>
+        <v>0.027</v>
       </c>
       <c r="F14" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>-0.086</v>
+        <v>0.027</v>
       </c>
       <c r="G14" s="66" t="n">
         <v>0.02</v>
       </c>
       <c r="H14" s="66" t="n">
         <f aca="false">G14+I14</f>
-        <v>-0.08</v>
+        <v>-0.043</v>
       </c>
       <c r="I14" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>-0.1</v>
+        <v>-0.063</v>
       </c>
       <c r="J14" s="66" t="n">
         <v>0.03</v>
       </c>
       <c r="K14" s="66" t="n">
         <f aca="false">J14+L14</f>
-        <v>0.086</v>
+        <v>-0.07</v>
       </c>
       <c r="L14" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>0.056</v>
+        <v>-0.1</v>
       </c>
       <c r="M14" s="66" t="n">
         <v>0.01</v>
       </c>
       <c r="N14" s="66" t="n">
         <f aca="false">M14+O14</f>
-        <v>-0.092</v>
+        <v>0.122</v>
       </c>
       <c r="O14" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>-0.102</v>
+        <v>0.112</v>
       </c>
       <c r="P14" s="66" t="n">
         <v>-0.01</v>
       </c>
       <c r="Q14" s="66" t="n">
         <f aca="false">P14+R14</f>
-        <v>0.05</v>
+        <v>0.026</v>
       </c>
       <c r="R14" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>0.06</v>
+        <v>0.036</v>
       </c>
       <c r="S14" s="66"/>
       <c r="T14" s="52" t="n">
@@ -13979,55 +14006,55 @@
       </c>
       <c r="E15" s="66" t="n">
         <f aca="false">D15+F15</f>
-        <v>-0.092</v>
+        <v>-0.111</v>
       </c>
       <c r="F15" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>0.008</v>
+        <v>-0.011</v>
       </c>
       <c r="G15" s="66" t="n">
         <v>-0.16</v>
       </c>
       <c r="H15" s="66" t="n">
         <f aca="false">G15+I15</f>
-        <v>-0.081</v>
+        <v>-0.052</v>
       </c>
       <c r="I15" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>0.079</v>
+        <v>0.108</v>
       </c>
       <c r="J15" s="66" t="n">
         <v>-0.21</v>
       </c>
       <c r="K15" s="66" t="n">
         <f aca="false">J15+L15</f>
-        <v>-0.293</v>
+        <v>-0.221</v>
       </c>
       <c r="L15" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>-0.083</v>
+        <v>-0.011</v>
       </c>
       <c r="M15" s="66" t="n">
         <v>-0.16</v>
       </c>
       <c r="N15" s="66" t="n">
         <f aca="false">M15+O15</f>
-        <v>-0.258</v>
+        <v>-0.14</v>
       </c>
       <c r="O15" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>-0.098</v>
+        <v>0.02</v>
       </c>
       <c r="P15" s="66" t="n">
         <v>-0.09</v>
       </c>
       <c r="Q15" s="66" t="n">
         <f aca="false">P15+R15</f>
-        <v>-0.107</v>
+        <v>-0.117</v>
       </c>
       <c r="R15" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>-0.017</v>
+        <v>-0.027</v>
       </c>
       <c r="S15" s="66"/>
       <c r="T15" s="52" t="n">
@@ -14050,55 +14077,55 @@
       </c>
       <c r="E16" s="66" t="n">
         <f aca="false">D16+F16</f>
-        <v>1.717</v>
+        <v>1.645</v>
       </c>
       <c r="F16" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>0.087</v>
+        <v>0.015</v>
       </c>
       <c r="G16" s="66" t="n">
         <v>0.76</v>
       </c>
       <c r="H16" s="66" t="n">
         <f aca="false">G16+I16</f>
-        <v>0.784</v>
+        <v>0.794</v>
       </c>
       <c r="I16" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>0.024</v>
+        <v>0.034</v>
       </c>
       <c r="J16" s="66" t="n">
         <v>0.85</v>
       </c>
       <c r="K16" s="66" t="n">
         <f aca="false">J16+L16</f>
-        <v>0.818</v>
+        <v>0.975</v>
       </c>
       <c r="L16" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>-0.032</v>
+        <v>0.125</v>
       </c>
       <c r="M16" s="66" t="n">
         <v>0.82</v>
       </c>
       <c r="N16" s="66" t="n">
         <f aca="false">M16+O16</f>
-        <v>0.908</v>
+        <v>0.743</v>
       </c>
       <c r="O16" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>0.088</v>
+        <v>-0.077</v>
       </c>
       <c r="P16" s="66" t="n">
         <v>1.54</v>
       </c>
       <c r="Q16" s="66" t="n">
         <f aca="false">P16+R16</f>
-        <v>1.499</v>
+        <v>1.51</v>
       </c>
       <c r="R16" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>-0.041</v>
+        <v>-0.03</v>
       </c>
       <c r="S16" s="66"/>
       <c r="T16" s="52" t="n">
@@ -14121,55 +14148,55 @@
       </c>
       <c r="E17" s="66" t="n">
         <f aca="false">D17+F17</f>
-        <v>1.828</v>
+        <v>1.846</v>
       </c>
       <c r="F17" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>0.068</v>
+        <v>0.086</v>
       </c>
       <c r="G17" s="66" t="n">
         <v>-0.25</v>
       </c>
       <c r="H17" s="66" t="n">
         <f aca="false">G17+I17</f>
-        <v>-0.165</v>
+        <v>-0.125</v>
       </c>
       <c r="I17" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>0.085</v>
+        <v>0.125</v>
       </c>
       <c r="J17" s="66" t="n">
         <v>-0.24</v>
       </c>
       <c r="K17" s="66" t="n">
         <f aca="false">J17+L17</f>
-        <v>-0.154</v>
+        <v>-0.288</v>
       </c>
       <c r="L17" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>0.086</v>
+        <v>-0.048</v>
       </c>
       <c r="M17" s="66" t="n">
         <v>-0.25</v>
       </c>
       <c r="N17" s="66" t="n">
         <f aca="false">M17+O17</f>
-        <v>-0.285</v>
+        <v>-0.247</v>
       </c>
       <c r="O17" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>-0.035</v>
+        <v>0.003</v>
       </c>
       <c r="P17" s="66" t="n">
         <v>-0.26</v>
       </c>
       <c r="Q17" s="66" t="n">
         <f aca="false">P17+R17</f>
-        <v>-0.291</v>
+        <v>-0.181</v>
       </c>
       <c r="R17" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>-0.031</v>
+        <v>0.079</v>
       </c>
       <c r="S17" s="66"/>
       <c r="T17" s="52" t="n">
@@ -14192,55 +14219,55 @@
       </c>
       <c r="E18" s="66" t="n">
         <f aca="false">D18+F18</f>
-        <v>-0.169</v>
+        <v>-0.319</v>
       </c>
       <c r="F18" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>0.091</v>
+        <v>-0.059</v>
       </c>
       <c r="G18" s="66" t="n">
         <v>-0.24</v>
       </c>
       <c r="H18" s="66" t="n">
         <f aca="false">G18+I18</f>
-        <v>-0.238</v>
+        <v>-0.169</v>
       </c>
       <c r="I18" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>0.002</v>
+        <v>0.071</v>
       </c>
       <c r="J18" s="66" t="n">
         <v>-0.23</v>
       </c>
       <c r="K18" s="66" t="n">
         <f aca="false">J18+L18</f>
-        <v>-0.159</v>
+        <v>-0.311</v>
       </c>
       <c r="L18" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>0.071</v>
+        <v>-0.081</v>
       </c>
       <c r="M18" s="66" t="n">
         <v>-0.19</v>
       </c>
       <c r="N18" s="66" t="n">
         <f aca="false">M18+O18</f>
-        <v>-0.268</v>
+        <v>-0.101</v>
       </c>
       <c r="O18" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>-0.078</v>
+        <v>0.089</v>
       </c>
       <c r="P18" s="66" t="n">
         <v>-0.14</v>
       </c>
       <c r="Q18" s="66" t="n">
         <f aca="false">P18+R18</f>
-        <v>-0.19</v>
+        <v>-0.096</v>
       </c>
       <c r="R18" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>-0.05</v>
+        <v>0.044</v>
       </c>
       <c r="S18" s="66"/>
       <c r="T18" s="52" t="n">
@@ -14263,55 +14290,55 @@
       </c>
       <c r="E19" s="66" t="n">
         <f aca="false">D19+F19</f>
-        <v>-0.336</v>
+        <v>-0.34</v>
       </c>
       <c r="F19" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>-0.076</v>
+        <v>-0.08</v>
       </c>
       <c r="G19" s="66" t="n">
         <v>-0.23</v>
       </c>
       <c r="H19" s="66" t="n">
         <f aca="false">G19+I19</f>
-        <v>-0.303</v>
+        <v>-0.213</v>
       </c>
       <c r="I19" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>-0.073</v>
+        <v>0.017</v>
       </c>
       <c r="J19" s="66" t="n">
         <v>-0.2</v>
       </c>
       <c r="K19" s="66" t="n">
         <f aca="false">J19+L19</f>
-        <v>-0.159</v>
+        <v>-0.125</v>
       </c>
       <c r="L19" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>0.041</v>
+        <v>0.075</v>
       </c>
       <c r="M19" s="66" t="n">
         <v>-0.15</v>
       </c>
       <c r="N19" s="66" t="n">
         <f aca="false">M19+O19</f>
-        <v>-0.254</v>
+        <v>-0.164</v>
       </c>
       <c r="O19" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>-0.104</v>
+        <v>-0.014</v>
       </c>
       <c r="P19" s="66" t="n">
         <v>-0.09</v>
       </c>
       <c r="Q19" s="66" t="n">
         <f aca="false">P19+R19</f>
-        <v>-0.168</v>
+        <v>-0.052</v>
       </c>
       <c r="R19" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>-0.078</v>
+        <v>0.038</v>
       </c>
       <c r="S19" s="66"/>
       <c r="T19" s="52" t="n">
@@ -14334,55 +14361,55 @@
       </c>
       <c r="E20" s="66" t="n">
         <f aca="false">D20+F20</f>
-        <v>-0.306</v>
+        <v>-0.192</v>
       </c>
       <c r="F20" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>-0.016</v>
+        <v>0.098</v>
       </c>
       <c r="G20" s="66" t="n">
         <v>-0.28</v>
       </c>
       <c r="H20" s="66" t="n">
         <f aca="false">G20+I20</f>
-        <v>-0.243</v>
+        <v>-0.272</v>
       </c>
       <c r="I20" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>0.037</v>
+        <v>0.008</v>
       </c>
       <c r="J20" s="66" t="n">
         <v>-0.27</v>
       </c>
       <c r="K20" s="66" t="n">
         <f aca="false">J20+L20</f>
-        <v>-0.326</v>
+        <v>-0.283</v>
       </c>
       <c r="L20" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>-0.056</v>
+        <v>-0.013</v>
       </c>
       <c r="M20" s="66" t="n">
         <v>-0.2</v>
       </c>
       <c r="N20" s="66" t="n">
         <f aca="false">M20+O20</f>
-        <v>-0.226</v>
+        <v>-0.282</v>
       </c>
       <c r="O20" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>-0.026</v>
+        <v>-0.082</v>
       </c>
       <c r="P20" s="66" t="n">
         <v>-0.11</v>
       </c>
       <c r="Q20" s="66" t="n">
         <f aca="false">P20+R20</f>
-        <v>-0.076</v>
+        <v>-0.09</v>
       </c>
       <c r="R20" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,125)/1000</f>
-        <v>0.034</v>
+        <v>0.02</v>
       </c>
       <c r="S20" s="66"/>
     </row>
@@ -14711,7 +14738,7 @@
     <row r="2" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="54" t="str">
         <f aca="false">"Kèm theo BBNT số: "&amp;VLOOKUP(W2,'Tuyến XB6A'!$A$2:$G$31,7,0)&amp;VLOOKUP(W2,'Tuyến XB6A'!$A$2:$G$31,4,0)</f>
-        <v>Kèm theo BBNT số: 02.NĐXB6A/CVXD ngày 15 tháng 08 năm 2026</v>
+        <v>Kèm theo BBNT số: 02.NĐXB6A/CVXD ngày 24 tháng 08 năm 2026</v>
       </c>
       <c r="B2" s="54"/>
       <c r="C2" s="54"/>
@@ -15117,55 +15144,55 @@
       </c>
       <c r="E25" s="67" t="n">
         <f aca="false">D25+F25</f>
-        <v>-6.938</v>
+        <v>-6.968</v>
       </c>
       <c r="F25" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>0.032</v>
+        <v>0.002</v>
       </c>
       <c r="G25" s="67" t="n">
         <v>-1.47</v>
       </c>
       <c r="H25" s="67" t="n">
         <f aca="false">G25+I25</f>
-        <v>-1.39</v>
+        <v>-1.477</v>
       </c>
       <c r="I25" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>0.08</v>
+        <v>-0.007</v>
       </c>
       <c r="J25" s="67" t="n">
         <v>-1.47</v>
       </c>
       <c r="K25" s="67" t="n">
         <f aca="false">J25+L25</f>
-        <v>-1.4</v>
+        <v>-1.44</v>
       </c>
       <c r="L25" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>0.07</v>
+        <v>0.03</v>
       </c>
       <c r="M25" s="67" t="n">
         <v>7.05</v>
       </c>
       <c r="N25" s="67" t="n">
         <f aca="false">M25+O25</f>
-        <v>7.067</v>
+        <v>6.947</v>
       </c>
       <c r="O25" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>0.017</v>
+        <v>-0.103</v>
       </c>
       <c r="P25" s="67" t="n">
         <v>-1.47</v>
       </c>
       <c r="Q25" s="67" t="n">
         <f aca="false">P25+R25</f>
-        <v>-1.516</v>
+        <v>-1.51</v>
       </c>
       <c r="R25" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>-0.046</v>
+        <v>-0.04</v>
       </c>
       <c r="S25" s="67" t="n">
         <f aca="false">ABS(D25)+ABS(M25)</f>
@@ -15173,11 +15200,11 @@
       </c>
       <c r="T25" s="67" t="n">
         <f aca="false">S25+U25</f>
-        <v>14.038</v>
+        <v>14.084</v>
       </c>
       <c r="U25" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,135)/1000</f>
-        <v>0.018</v>
+        <v>0.064</v>
       </c>
       <c r="V25" s="85"/>
     </row>
@@ -15199,55 +15226,55 @@
       </c>
       <c r="E26" s="67" t="n">
         <f aca="false">D26+F26</f>
-        <v>-6.931</v>
+        <v>-6.962</v>
       </c>
       <c r="F26" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>0.109</v>
+        <v>0.078</v>
       </c>
       <c r="G26" s="67" t="n">
         <v>-1.51</v>
       </c>
       <c r="H26" s="67" t="n">
         <f aca="false">G26+I26</f>
-        <v>-1.561</v>
+        <v>-1.455</v>
       </c>
       <c r="I26" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>-0.051</v>
+        <v>0.055</v>
       </c>
       <c r="J26" s="67" t="n">
         <v>-1.51</v>
       </c>
       <c r="K26" s="67" t="n">
         <f aca="false">J26+L26</f>
-        <v>-1.463</v>
+        <v>-1.477</v>
       </c>
       <c r="L26" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>0.047</v>
+        <v>0.033</v>
       </c>
       <c r="M26" s="67" t="n">
         <v>7.09</v>
       </c>
       <c r="N26" s="67" t="n">
         <f aca="false">M26+O26</f>
-        <v>7.145</v>
+        <v>7.091</v>
       </c>
       <c r="O26" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>0.055</v>
+        <v>0.001</v>
       </c>
       <c r="P26" s="67" t="n">
         <v>-1.51</v>
       </c>
       <c r="Q26" s="67" t="n">
         <f aca="false">P26+R26</f>
-        <v>-1.481</v>
+        <v>-1.467</v>
       </c>
       <c r="R26" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>0.029</v>
+        <v>0.043</v>
       </c>
       <c r="S26" s="67" t="n">
         <f aca="false">ABS(D26)+ABS(M26)</f>
@@ -15255,11 +15282,11 @@
       </c>
       <c r="T26" s="67" t="n">
         <f aca="false">S26+U26</f>
-        <v>14.197</v>
+        <v>14.233</v>
       </c>
       <c r="U26" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,135)/1000</f>
-        <v>0.067</v>
+        <v>0.103</v>
       </c>
       <c r="V26" s="85"/>
     </row>
@@ -15281,55 +15308,55 @@
       </c>
       <c r="E27" s="67" t="n">
         <f aca="false">D27+F27</f>
-        <v>-7.337</v>
+        <v>-7.211</v>
       </c>
       <c r="F27" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>-0.057</v>
+        <v>0.069</v>
       </c>
       <c r="G27" s="67" t="n">
         <v>-1.56</v>
       </c>
       <c r="H27" s="67" t="n">
         <f aca="false">G27+I27</f>
-        <v>-1.589</v>
+        <v>-1.538</v>
       </c>
       <c r="I27" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>-0.029</v>
+        <v>0.022</v>
       </c>
       <c r="J27" s="67" t="n">
         <v>-1.56</v>
       </c>
       <c r="K27" s="67" t="n">
         <f aca="false">J27+L27</f>
-        <v>-1.613</v>
+        <v>-1.643</v>
       </c>
       <c r="L27" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>-0.053</v>
+        <v>-0.083</v>
       </c>
       <c r="M27" s="67" t="n">
         <v>7.26</v>
       </c>
       <c r="N27" s="67" t="n">
         <f aca="false">M27+O27</f>
-        <v>7.345</v>
+        <v>7.23</v>
       </c>
       <c r="O27" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>0.085</v>
+        <v>-0.03</v>
       </c>
       <c r="P27" s="67" t="n">
         <v>-1.56</v>
       </c>
       <c r="Q27" s="67" t="n">
         <f aca="false">P27+R27</f>
-        <v>-1.583</v>
+        <v>-1.571</v>
       </c>
       <c r="R27" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>-0.023</v>
+        <v>-0.011</v>
       </c>
       <c r="S27" s="67" t="n">
         <f aca="false">ABS(D27)+ABS(M27)</f>
@@ -15337,11 +15364,11 @@
       </c>
       <c r="T27" s="67" t="n">
         <f aca="false">S27+U27</f>
-        <v>14.573</v>
+        <v>14.559</v>
       </c>
       <c r="U27" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,135)/1000</f>
-        <v>0.033</v>
+        <v>0.019</v>
       </c>
       <c r="V27" s="85"/>
     </row>
@@ -15396,55 +15423,55 @@
       </c>
       <c r="E29" s="67" t="n">
         <f aca="false">D29+F29</f>
-        <v>-4.827</v>
+        <v>-4.836</v>
       </c>
       <c r="F29" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>-0.007</v>
+        <v>-0.016</v>
       </c>
       <c r="G29" s="67" t="n">
         <v>-1.63</v>
       </c>
       <c r="H29" s="67" t="n">
         <f aca="false">G29+I29</f>
-        <v>-1.646</v>
+        <v>-1.669</v>
       </c>
       <c r="I29" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>-0.016</v>
+        <v>-0.039</v>
       </c>
       <c r="J29" s="67" t="n">
         <v>-1.63</v>
       </c>
       <c r="K29" s="67" t="n">
         <f aca="false">J29+L29</f>
-        <v>-1.618</v>
+        <v>-1.522</v>
       </c>
       <c r="L29" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>0.012</v>
+        <v>0.108</v>
       </c>
       <c r="M29" s="67" t="n">
         <v>7.68</v>
       </c>
       <c r="N29" s="67" t="n">
         <f aca="false">M29+O29</f>
-        <v>7.745</v>
+        <v>7.692</v>
       </c>
       <c r="O29" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>0.065</v>
+        <v>0.012</v>
       </c>
       <c r="P29" s="67" t="n">
         <v>-1.63</v>
       </c>
       <c r="Q29" s="67" t="n">
         <f aca="false">P29+R29</f>
-        <v>-1.523</v>
+        <v>-1.697</v>
       </c>
       <c r="R29" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>0.107</v>
+        <v>-0.067</v>
       </c>
       <c r="S29" s="67" t="n">
         <f aca="false">ABS(D29)+ABS(M29)</f>
@@ -15452,11 +15479,11 @@
       </c>
       <c r="T29" s="67" t="n">
         <f aca="false">S29+U29</f>
-        <v>12.465</v>
+        <v>12.56</v>
       </c>
       <c r="U29" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,135)/1000</f>
-        <v>-0.035</v>
+        <v>0.06</v>
       </c>
       <c r="V29" s="85"/>
     </row>
@@ -15478,55 +15505,55 @@
       </c>
       <c r="E30" s="67" t="n">
         <f aca="false">D30+F30</f>
-        <v>-7.661</v>
+        <v>-7.748</v>
       </c>
       <c r="F30" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>-0.011</v>
+        <v>-0.098</v>
       </c>
       <c r="G30" s="67" t="n">
         <v>-1.68</v>
       </c>
       <c r="H30" s="67" t="n">
         <f aca="false">G30+I30</f>
-        <v>-1.683</v>
+        <v>-1.752</v>
       </c>
       <c r="I30" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>-0.003</v>
+        <v>-0.072</v>
       </c>
       <c r="J30" s="67" t="n">
         <v>-1.68</v>
       </c>
       <c r="K30" s="67" t="n">
         <f aca="false">J30+L30</f>
-        <v>-1.621</v>
+        <v>-1.709</v>
       </c>
       <c r="L30" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>0.059</v>
+        <v>-0.029</v>
       </c>
       <c r="M30" s="67" t="n">
         <v>7.32</v>
       </c>
       <c r="N30" s="67" t="n">
         <f aca="false">M30+O30</f>
-        <v>7.263</v>
+        <v>7.276</v>
       </c>
       <c r="O30" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>-0.057</v>
+        <v>-0.044</v>
       </c>
       <c r="P30" s="67" t="n">
         <v>-1.68</v>
       </c>
       <c r="Q30" s="67" t="n">
         <f aca="false">P30+R30</f>
-        <v>-1.6</v>
+        <v>-1.65</v>
       </c>
       <c r="R30" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>0.08</v>
+        <v>0.03</v>
       </c>
       <c r="S30" s="67" t="n">
         <f aca="false">ABS(D30)+ABS(M30)</f>
@@ -15534,11 +15561,11 @@
       </c>
       <c r="T30" s="67" t="n">
         <f aca="false">S30+U30</f>
-        <v>15.098</v>
+        <v>14.865</v>
       </c>
       <c r="U30" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,135)/1000</f>
-        <v>0.128</v>
+        <v>-0.105</v>
       </c>
       <c r="V30" s="85"/>
     </row>
@@ -15560,55 +15587,55 @@
       </c>
       <c r="E31" s="67" t="n">
         <f aca="false">D31+F31</f>
-        <v>-7.665</v>
+        <v>-7.698</v>
       </c>
       <c r="F31" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>-0.035</v>
+        <v>-0.068</v>
       </c>
       <c r="G31" s="67" t="n">
         <v>-1.73</v>
       </c>
       <c r="H31" s="67" t="n">
         <f aca="false">G31+I31</f>
-        <v>-1.8</v>
+        <v>-1.804</v>
       </c>
       <c r="I31" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>-0.07</v>
+        <v>-0.074</v>
       </c>
       <c r="J31" s="67" t="n">
         <v>-1.73</v>
       </c>
       <c r="K31" s="67" t="n">
         <f aca="false">J31+L31</f>
-        <v>-1.66</v>
+        <v>-1.757</v>
       </c>
       <c r="L31" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>0.07</v>
+        <v>-0.027</v>
       </c>
       <c r="M31" s="67" t="n">
         <v>7.15</v>
       </c>
       <c r="N31" s="67" t="n">
         <f aca="false">M31+O31</f>
-        <v>7.194</v>
+        <v>7.239</v>
       </c>
       <c r="O31" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>0.044</v>
+        <v>0.089</v>
       </c>
       <c r="P31" s="67" t="n">
         <v>-1.73</v>
       </c>
       <c r="Q31" s="67" t="n">
         <f aca="false">P31+R31</f>
-        <v>-1.806</v>
+        <v>-1.762</v>
       </c>
       <c r="R31" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,115)/1000</f>
-        <v>-0.076</v>
+        <v>-0.032</v>
       </c>
       <c r="S31" s="67" t="n">
         <f aca="false">ABS(D31)+ABS(M31)</f>
@@ -15616,11 +15643,11 @@
       </c>
       <c r="T31" s="67" t="n">
         <f aca="false">S31+U31</f>
-        <v>14.84</v>
+        <v>14.899</v>
       </c>
       <c r="U31" s="67" t="n">
         <f aca="false">RANDBETWEEN(-105,135)/1000</f>
-        <v>0.06</v>
+        <v>0.119</v>
       </c>
       <c r="V31" s="85"/>
     </row>
@@ -15832,7 +15859,7 @@
     <row r="2" s="90" customFormat="true" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="91" t="str">
         <f aca="false">"Kèm theo BBNT số: "&amp;VLOOKUP(N2,'Tuyến XB6A'!$A$2:$G$29,7,0)&amp;VLOOKUP(N2,'Tuyến XB6A'!$A$2:$G$29,4,0)</f>
-        <v>Kèm theo BBNT số: 02.NĐXB6A/CVXD ngày 15 tháng 08 năm 2026</v>
+        <v>Kèm theo BBNT số: 02.NĐXB6A/CVXD ngày 24 tháng 08 năm 2026</v>
       </c>
       <c r="B2" s="91"/>
       <c r="C2" s="91"/>
@@ -17090,7 +17117,7 @@
       <c r="I12" s="108"/>
       <c r="J12" s="109" t="n">
         <f aca="false">(G12+G13)*D12/2</f>
-        <v>406.32805</v>
+        <v>406.67145</v>
       </c>
       <c r="K12" s="109"/>
       <c r="L12" s="109"/>
@@ -17115,20 +17142,20 @@
       </c>
       <c r="E13" s="67" t="n">
         <f aca="false">RANDBETWEEN(1,7)/100</f>
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="F13" s="108" t="n">
         <v>23.91</v>
       </c>
       <c r="G13" s="108" t="n">
         <f aca="false">+F13+E13</f>
-        <v>23.92</v>
+        <v>23.96</v>
       </c>
       <c r="H13" s="108"/>
       <c r="I13" s="108"/>
       <c r="J13" s="109" t="n">
         <f aca="false">(G13+G14)*D13/2</f>
-        <v>399.2632</v>
+        <v>399.7786</v>
       </c>
       <c r="K13" s="109"/>
       <c r="L13" s="109"/>
@@ -17153,20 +17180,20 @@
       </c>
       <c r="E14" s="67" t="n">
         <f aca="false">RANDBETWEEN(1,7)/100</f>
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="F14" s="108" t="n">
         <v>22.53</v>
       </c>
       <c r="G14" s="108" t="n">
         <f aca="false">+F14+E14</f>
-        <v>22.56</v>
+        <v>22.58</v>
       </c>
       <c r="H14" s="108"/>
       <c r="I14" s="108"/>
       <c r="J14" s="109" t="n">
         <f aca="false">(G14+G15)*D14/2</f>
-        <v>146.3016</v>
+        <v>146.4313</v>
       </c>
       <c r="K14" s="109"/>
       <c r="L14" s="109"/>
@@ -17198,7 +17225,7 @@
       <c r="I15" s="108"/>
       <c r="J15" s="109" t="n">
         <f aca="false">(G15+G16)*D15/2</f>
-        <v>109.737</v>
+        <v>109.6302</v>
       </c>
       <c r="K15" s="109"/>
       <c r="L15" s="109"/>
@@ -17223,20 +17250,20 @@
       </c>
       <c r="E16" s="67" t="n">
         <f aca="false">RANDBETWEEN(1,7)/100</f>
-        <v>0.04</v>
+        <v>0.02</v>
       </c>
       <c r="F16" s="108" t="n">
         <v>20.51</v>
       </c>
       <c r="G16" s="108" t="n">
         <f aca="false">+F16+E16</f>
-        <v>20.55</v>
+        <v>20.53</v>
       </c>
       <c r="H16" s="108"/>
       <c r="I16" s="108"/>
       <c r="J16" s="109" t="n">
         <f aca="false">(G16+G17)*D16/2</f>
-        <v>383.14855</v>
+        <v>382.97685</v>
       </c>
       <c r="K16" s="109"/>
       <c r="L16" s="109"/>
@@ -17274,7 +17301,7 @@
       <c r="I17" s="108"/>
       <c r="J17" s="109" t="n">
         <f aca="false">(G17+G18)*D17/2</f>
-        <v>422.81125</v>
+        <v>422.382</v>
       </c>
       <c r="K17" s="109"/>
       <c r="L17" s="109"/>
@@ -17299,20 +17326,20 @@
       </c>
       <c r="E18" s="67" t="n">
         <f aca="false">RANDBETWEEN(1,7)/100</f>
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="F18" s="108" t="n">
         <v>25.11</v>
       </c>
       <c r="G18" s="108" t="n">
         <f aca="false">+F18+E18</f>
-        <v>25.17</v>
+        <v>25.12</v>
       </c>
       <c r="H18" s="108"/>
       <c r="I18" s="108"/>
       <c r="J18" s="109" t="n">
         <f aca="false">(G18+G19)*D18/2</f>
-        <v>182.35665</v>
+        <v>181.9944</v>
       </c>
       <c r="K18" s="109"/>
       <c r="L18" s="109"/>
@@ -17359,7 +17386,7 @@
       <c r="I20" s="113"/>
       <c r="J20" s="114" t="n">
         <f aca="false">SUM(J11:J19)</f>
-        <v>2279.71545</v>
+        <v>2279.63395</v>
       </c>
       <c r="K20" s="114"/>
       <c r="L20" s="114"/>
@@ -19387,7 +19414,7 @@
     <row r="2" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="54" t="str">
         <f aca="false">"Kèm theo BBNT số: "&amp;VLOOKUP(W2,'Tuyến XB6A'!$A$2:$G$31,7,0)&amp;VLOOKUP(W2,'Tuyến XB6A'!$A$2:$G$31,4,0)</f>
-        <v>Kèm theo BBNT số: 03.NĐXB6A/CVXD ngày 15 tháng 08 năm 2026</v>
+        <v>Kèm theo BBNT số: 03.NĐXB6A/CVXD ngày 24 tháng 08 năm 2026</v>
       </c>
       <c r="B2" s="54"/>
       <c r="C2" s="54"/>
@@ -19798,33 +19825,33 @@
       </c>
       <c r="E25" s="67" t="n">
         <f aca="false">+D25+F25</f>
-        <v>2.06</v>
+        <v>2.09</v>
       </c>
       <c r="F25" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.06</v>
+        <v>0.09</v>
       </c>
       <c r="G25" s="67" t="n">
         <v>1.41</v>
       </c>
       <c r="H25" s="67" t="n">
         <f aca="false">+G25+I25</f>
-        <v>1.47</v>
+        <v>1.51</v>
       </c>
       <c r="I25" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="J25" s="67" t="n">
         <v>6.97</v>
       </c>
       <c r="K25" s="67" t="n">
         <f aca="false">+J25+L25</f>
-        <v>7.03</v>
+        <v>7.05</v>
       </c>
       <c r="L25" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="M25" s="67" t="n">
         <v>7.05</v>
@@ -19842,11 +19869,11 @@
       </c>
       <c r="Q25" s="67" t="n">
         <f aca="false">+P25+R25</f>
-        <v>1.5</v>
+        <v>1.47</v>
       </c>
       <c r="R25" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.09</v>
+        <v>0.06</v>
       </c>
       <c r="S25" s="67" t="n">
         <v>2</v>
@@ -19879,11 +19906,11 @@
       </c>
       <c r="E26" s="67" t="n">
         <f aca="false">+D26+F26</f>
-        <v>2.07</v>
+        <v>2.05</v>
       </c>
       <c r="F26" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.07</v>
+        <v>0.05</v>
       </c>
       <c r="G26" s="67" t="n">
         <v>1.41</v>
@@ -19901,44 +19928,44 @@
       </c>
       <c r="K26" s="67" t="n">
         <f aca="false">+J26+L26</f>
-        <v>7.14</v>
+        <v>7.13</v>
       </c>
       <c r="L26" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="M26" s="67" t="n">
         <v>7.09</v>
       </c>
       <c r="N26" s="67" t="n">
         <f aca="false">+M26+O26</f>
-        <v>7.14</v>
+        <v>7.15</v>
       </c>
       <c r="O26" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="P26" s="67" t="n">
         <v>1.41</v>
       </c>
       <c r="Q26" s="67" t="n">
         <f aca="false">+P26+R26</f>
-        <v>1.51</v>
+        <v>1.46</v>
       </c>
       <c r="R26" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="S26" s="67" t="n">
         <v>2</v>
       </c>
       <c r="T26" s="67" t="n">
         <f aca="false">+S26+U26</f>
-        <v>2.08</v>
+        <v>2.07</v>
       </c>
       <c r="U26" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.08</v>
+        <v>0.07</v>
       </c>
       <c r="V26" s="85"/>
     </row>
@@ -19960,66 +19987,66 @@
       </c>
       <c r="E27" s="67" t="n">
         <f aca="false">+D27+F27</f>
-        <v>2.05</v>
+        <v>2.1</v>
       </c>
       <c r="F27" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="G27" s="67" t="n">
         <v>1.41</v>
       </c>
       <c r="H27" s="67" t="n">
         <f aca="false">+G27+I27</f>
-        <v>1.46</v>
+        <v>1.47</v>
       </c>
       <c r="I27" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="J27" s="67" t="n">
         <v>7.28</v>
       </c>
       <c r="K27" s="67" t="n">
         <f aca="false">+J27+L27</f>
-        <v>7.35</v>
+        <v>7.33</v>
       </c>
       <c r="L27" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.07</v>
+        <v>0.05</v>
       </c>
       <c r="M27" s="67" t="n">
         <v>7.26</v>
       </c>
       <c r="N27" s="67" t="n">
         <f aca="false">+M27+O27</f>
-        <v>7.35</v>
+        <v>7.32</v>
       </c>
       <c r="O27" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.09</v>
+        <v>0.06</v>
       </c>
       <c r="P27" s="67" t="n">
         <v>1.41</v>
       </c>
       <c r="Q27" s="67" t="n">
         <f aca="false">+P27+R27</f>
-        <v>1.5</v>
+        <v>1.49</v>
       </c>
       <c r="R27" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="S27" s="67" t="n">
         <v>2</v>
       </c>
       <c r="T27" s="67" t="n">
         <f aca="false">+S27+U27</f>
-        <v>2.08</v>
+        <v>2.09</v>
       </c>
       <c r="U27" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.08</v>
+        <v>0.09</v>
       </c>
       <c r="V27" s="85"/>
     </row>
@@ -20074,11 +20101,11 @@
       </c>
       <c r="E29" s="67" t="n">
         <f aca="false">+D29+F29</f>
-        <v>2.07</v>
+        <v>2.09</v>
       </c>
       <c r="F29" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.07</v>
+        <v>0.09</v>
       </c>
       <c r="G29" s="67" t="n">
         <v>1.41</v>
@@ -20096,44 +20123,44 @@
       </c>
       <c r="K29" s="67" t="n">
         <f aca="false">+J29+L29</f>
-        <v>4.92</v>
+        <v>4.89</v>
       </c>
       <c r="L29" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.1</v>
+        <v>0.07</v>
       </c>
       <c r="M29" s="67" t="n">
         <v>7.68</v>
       </c>
       <c r="N29" s="67" t="n">
         <f aca="false">+M29+O29</f>
-        <v>7.74</v>
+        <v>7.77</v>
       </c>
       <c r="O29" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.06</v>
+        <v>0.09</v>
       </c>
       <c r="P29" s="67" t="n">
         <v>1.41</v>
       </c>
       <c r="Q29" s="67" t="n">
         <f aca="false">+P29+R29</f>
-        <v>1.49</v>
+        <v>1.51</v>
       </c>
       <c r="R29" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="S29" s="67" t="n">
         <v>2</v>
       </c>
       <c r="T29" s="67" t="n">
         <f aca="false">+S29+U29</f>
-        <v>2.07</v>
+        <v>2.05</v>
       </c>
       <c r="U29" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.07</v>
+        <v>0.05</v>
       </c>
       <c r="V29" s="85"/>
     </row>
@@ -20155,22 +20182,22 @@
       </c>
       <c r="E30" s="67" t="n">
         <f aca="false">+D30+F30</f>
-        <v>2.07</v>
+        <v>2.05</v>
       </c>
       <c r="F30" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.07</v>
+        <v>0.05</v>
       </c>
       <c r="G30" s="67" t="n">
         <v>1.41</v>
       </c>
       <c r="H30" s="67" t="n">
         <f aca="false">+G30+I30</f>
-        <v>1.46</v>
+        <v>1.48</v>
       </c>
       <c r="I30" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.05</v>
+        <v>0.07</v>
       </c>
       <c r="J30" s="67" t="n">
         <v>7.65</v>
@@ -20188,33 +20215,33 @@
       </c>
       <c r="N30" s="67" t="n">
         <f aca="false">+M30+O30</f>
-        <v>7.39</v>
+        <v>7.42</v>
       </c>
       <c r="O30" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.07</v>
+        <v>0.1</v>
       </c>
       <c r="P30" s="67" t="n">
         <v>1.41</v>
       </c>
       <c r="Q30" s="67" t="n">
         <f aca="false">+P30+R30</f>
-        <v>1.47</v>
+        <v>1.48</v>
       </c>
       <c r="R30" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.06</v>
+        <v>0.07</v>
       </c>
       <c r="S30" s="67" t="n">
         <v>2</v>
       </c>
       <c r="T30" s="67" t="n">
         <f aca="false">+S30+U30</f>
-        <v>2.07</v>
+        <v>2.06</v>
       </c>
       <c r="U30" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.07</v>
+        <v>0.06</v>
       </c>
       <c r="V30" s="85"/>
     </row>
@@ -20236,66 +20263,66 @@
       </c>
       <c r="E31" s="67" t="n">
         <f aca="false">+D31+F31</f>
-        <v>2.1</v>
+        <v>2.05</v>
       </c>
       <c r="F31" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="G31" s="67" t="n">
         <v>1.41</v>
       </c>
       <c r="H31" s="67" t="n">
         <f aca="false">+G31+I31</f>
-        <v>1.5</v>
+        <v>1.49</v>
       </c>
       <c r="I31" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="J31" s="67" t="n">
         <v>7.63</v>
       </c>
       <c r="K31" s="67" t="n">
         <f aca="false">+J31+L31</f>
-        <v>7.72</v>
+        <v>7.71</v>
       </c>
       <c r="L31" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="M31" s="67" t="n">
         <v>7.15</v>
       </c>
       <c r="N31" s="67" t="n">
         <f aca="false">+M31+O31</f>
-        <v>7.21</v>
+        <v>7.2</v>
       </c>
       <c r="O31" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="P31" s="67" t="n">
         <v>1.41</v>
       </c>
       <c r="Q31" s="67" t="n">
         <f aca="false">+P31+R31</f>
-        <v>1.46</v>
+        <v>1.5</v>
       </c>
       <c r="R31" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.05</v>
+        <v>0.09</v>
       </c>
       <c r="S31" s="67" t="n">
         <v>2</v>
       </c>
       <c r="T31" s="67" t="n">
         <f aca="false">+S31+U31</f>
-        <v>2.1</v>
+        <v>2.06</v>
       </c>
       <c r="U31" s="67" t="n">
         <f aca="false">RANDBETWEEN(5,10)/100</f>
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="V31" s="85"/>
     </row>
@@ -20534,7 +20561,7 @@
     <row r="2" s="90" customFormat="true" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="91" t="str">
         <f aca="false">"Kèm theo BBNT số: "&amp;VLOOKUP(O2,'Tuyến XB6A'!$A$2:$G$29,7,0)&amp;VLOOKUP(O2,'Tuyến XB6A'!$A$2:$G$29,4,0)</f>
-        <v>Kèm theo BBNT số: 03.NĐXB6A/CVXD ngày 15 tháng 08 năm 2026</v>
+        <v>Kèm theo BBNT số: 03.NĐXB6A/CVXD ngày 24 tháng 08 năm 2026</v>
       </c>
       <c r="B2" s="91"/>
       <c r="C2" s="91"/>
@@ -21745,7 +21772,7 @@
       </c>
       <c r="L11" s="109" t="n">
         <f aca="false">(K11+K12)*D11/2</f>
-        <v>208.37245</v>
+        <v>208.96135</v>
       </c>
       <c r="M11" s="110"/>
       <c r="O11" s="136"/>
@@ -21769,15 +21796,15 @@
       </c>
       <c r="E12" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!E25</f>
-        <v>2.06</v>
+        <v>2.09</v>
       </c>
       <c r="F12" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!H25</f>
-        <v>1.47</v>
+        <v>1.51</v>
       </c>
       <c r="G12" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!K25</f>
-        <v>7.03</v>
+        <v>7.05</v>
       </c>
       <c r="H12" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!N25</f>
@@ -21785,7 +21812,7 @@
       </c>
       <c r="I12" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!Q25</f>
-        <v>1.5</v>
+        <v>1.47</v>
       </c>
       <c r="J12" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!T25</f>
@@ -21793,11 +21820,11 @@
       </c>
       <c r="K12" s="135" t="n">
         <f aca="false">SUM(E12:J12)</f>
-        <v>21.23</v>
+        <v>21.29</v>
       </c>
       <c r="L12" s="109" t="n">
         <f aca="false">(K12+K13)*D12/2</f>
-        <v>366.32195</v>
+        <v>366.15025</v>
       </c>
       <c r="M12" s="110"/>
       <c r="O12" s="136"/>
@@ -21821,7 +21848,7 @@
       </c>
       <c r="E13" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!E26</f>
-        <v>2.07</v>
+        <v>2.05</v>
       </c>
       <c r="F13" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!H26</f>
@@ -21829,27 +21856,27 @@
       </c>
       <c r="G13" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!K26</f>
-        <v>7.14</v>
+        <v>7.13</v>
       </c>
       <c r="H13" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!N26</f>
-        <v>7.14</v>
+        <v>7.15</v>
       </c>
       <c r="I13" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!Q26</f>
-        <v>1.51</v>
+        <v>1.46</v>
       </c>
       <c r="J13" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!T26</f>
-        <v>2.08</v>
+        <v>2.07</v>
       </c>
       <c r="K13" s="135" t="n">
         <f aca="false">SUM(E13:J13)</f>
-        <v>21.44</v>
+        <v>21.36</v>
       </c>
       <c r="L13" s="109" t="n">
         <f aca="false">(K13+K14)*D13/2</f>
-        <v>371.3457</v>
+        <v>370.7444</v>
       </c>
       <c r="M13" s="110"/>
       <c r="O13" s="136"/>
@@ -21873,35 +21900,35 @@
       </c>
       <c r="E14" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!E27</f>
-        <v>2.05</v>
+        <v>2.1</v>
       </c>
       <c r="F14" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!H27</f>
-        <v>1.46</v>
+        <v>1.47</v>
       </c>
       <c r="G14" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!K27</f>
-        <v>7.35</v>
+        <v>7.33</v>
       </c>
       <c r="H14" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!N27</f>
-        <v>7.35</v>
+        <v>7.32</v>
       </c>
       <c r="I14" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!Q27</f>
-        <v>1.5</v>
+        <v>1.49</v>
       </c>
       <c r="J14" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!T27</f>
-        <v>2.08</v>
+        <v>2.09</v>
       </c>
       <c r="K14" s="135" t="n">
         <f aca="false">SUM(E14:J14)</f>
-        <v>21.79</v>
+        <v>21.8</v>
       </c>
       <c r="L14" s="109" t="n">
         <f aca="false">(K14+K15)*D14/2</f>
-        <v>141.30815</v>
+        <v>141.373</v>
       </c>
       <c r="M14" s="110"/>
       <c r="O14" s="136"/>
@@ -21935,7 +21962,7 @@
       </c>
       <c r="L15" s="109" t="n">
         <f aca="false">(K15+K16)*D15/2</f>
-        <v>105.5184</v>
+        <v>105.6252</v>
       </c>
       <c r="M15" s="110"/>
       <c r="O15" s="136"/>
@@ -21959,7 +21986,7 @@
       </c>
       <c r="E16" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!E29</f>
-        <v>2.07</v>
+        <v>2.09</v>
       </c>
       <c r="F16" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!H29</f>
@@ -21967,27 +21994,27 @@
       </c>
       <c r="G16" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!K29</f>
-        <v>4.92</v>
+        <v>4.89</v>
       </c>
       <c r="H16" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!N29</f>
-        <v>7.74</v>
+        <v>7.77</v>
       </c>
       <c r="I16" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!Q29</f>
-        <v>1.49</v>
+        <v>1.51</v>
       </c>
       <c r="J16" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!T29</f>
-        <v>2.07</v>
+        <v>2.05</v>
       </c>
       <c r="K16" s="135" t="n">
         <f aca="false">SUM(E16:J16)</f>
-        <v>19.76</v>
+        <v>19.78</v>
       </c>
       <c r="L16" s="109" t="n">
         <f aca="false">(K16+K17)*D16/2</f>
-        <v>360.2266</v>
+        <v>360.65585</v>
       </c>
       <c r="M16" s="110"/>
       <c r="O16" s="136"/>
@@ -22011,11 +22038,11 @@
       </c>
       <c r="E17" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!E30</f>
-        <v>2.07</v>
+        <v>2.05</v>
       </c>
       <c r="F17" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!H30</f>
-        <v>1.46</v>
+        <v>1.48</v>
       </c>
       <c r="G17" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!K30</f>
@@ -22023,23 +22050,23 @@
       </c>
       <c r="H17" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!N30</f>
-        <v>7.39</v>
+        <v>7.42</v>
       </c>
       <c r="I17" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!Q30</f>
-        <v>1.47</v>
+        <v>1.48</v>
       </c>
       <c r="J17" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!T30</f>
-        <v>2.07</v>
+        <v>2.06</v>
       </c>
       <c r="K17" s="135" t="n">
         <f aca="false">SUM(E17:J17)</f>
-        <v>22.2</v>
+        <v>22.23</v>
       </c>
       <c r="L17" s="109" t="n">
         <f aca="false">(K17+K18)*D17/2</f>
-        <v>380.22965</v>
+        <v>379.8004</v>
       </c>
       <c r="M17" s="110"/>
       <c r="O17" s="136"/>
@@ -22063,35 +22090,35 @@
       </c>
       <c r="E18" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!E31</f>
-        <v>2.1</v>
+        <v>2.05</v>
       </c>
       <c r="F18" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!H31</f>
-        <v>1.5</v>
+        <v>1.49</v>
       </c>
       <c r="G18" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!K31</f>
-        <v>7.72</v>
+        <v>7.71</v>
       </c>
       <c r="H18" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!N31</f>
-        <v>7.21</v>
+        <v>7.2</v>
       </c>
       <c r="I18" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!Q31</f>
-        <v>1.46</v>
+        <v>1.5</v>
       </c>
       <c r="J18" s="134" t="n">
         <f aca="false">'3. KTHH vải lọc'!T31</f>
-        <v>2.1</v>
+        <v>2.06</v>
       </c>
       <c r="K18" s="135" t="n">
         <f aca="false">SUM(E18:J18)</f>
-        <v>22.09</v>
+        <v>22.01</v>
       </c>
       <c r="L18" s="109" t="n">
         <f aca="false">(K18+K19)*D18/2</f>
-        <v>160.04205</v>
+        <v>159.46245</v>
       </c>
       <c r="M18" s="110"/>
       <c r="O18" s="136"/>
@@ -22141,7 +22168,7 @@
       <c r="K20" s="113"/>
       <c r="L20" s="114" t="n">
         <f aca="false">SUM(L11:L19)</f>
-        <v>2093.36495</v>
+        <v>2092.7729</v>
       </c>
       <c r="M20" s="115"/>
       <c r="O20" s="138"/>
@@ -24664,7 +24691,7 @@
     <row r="2" s="145" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="144" t="str">
         <f aca="false">"Kèm theo BBNT số: "&amp;VLOOKUP(L2,'Tuyến XB6A'!$A$2:$G$31,7,0)&amp;VLOOKUP(L2,'Tuyến XB6A'!$A$2:$G$31,4,0)</f>
-        <v>Kèm theo BBNT số: 26.NĐXB6A/CVXD ngày 10 tháng 09 năm 2026</v>
+        <v>Kèm theo BBNT số: 26.NĐXB6A/CVXD ngày 13 tháng 09 năm 2026</v>
       </c>
       <c r="B2" s="144"/>
       <c r="C2" s="144"/>
@@ -25854,11 +25881,11 @@
       </c>
       <c r="F11" s="134" t="n">
         <f aca="false">+E11+G11</f>
-        <v>7.478</v>
+        <v>7.507</v>
       </c>
       <c r="G11" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,110)/1000</f>
-        <v>-0.022</v>
+        <v>0.007</v>
       </c>
       <c r="H11" s="109" t="n">
         <f aca="false">+(E11+E12)/2*D11</f>
@@ -25866,11 +25893,11 @@
       </c>
       <c r="I11" s="109" t="n">
         <f aca="false">+(F11+F12)/2*D11</f>
-        <v>147.93168</v>
+        <v>147.077775</v>
       </c>
       <c r="J11" s="109" t="n">
         <f aca="false">+I11-H11</f>
-        <v>0.706679999999977</v>
+        <v>-0.14722500000002</v>
       </c>
       <c r="K11" s="110"/>
       <c r="L11" s="136"/>
@@ -25896,11 +25923,11 @@
       </c>
       <c r="F12" s="134" t="n">
         <f aca="false">+E12+G12</f>
-        <v>7.594</v>
+        <v>7.478</v>
       </c>
       <c r="G12" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,110)/1000</f>
-        <v>0.094</v>
+        <v>-0.022</v>
       </c>
       <c r="H12" s="109" t="n">
         <f aca="false">+(E12+E13)/2*D12</f>
@@ -25908,11 +25935,11 @@
       </c>
       <c r="I12" s="109" t="n">
         <f aca="false">+(F12+F13)/2*D12</f>
-        <v>130.431905</v>
+        <v>128.886605</v>
       </c>
       <c r="J12" s="109" t="n">
         <f aca="false">+I12-H12</f>
-        <v>1.65690500000002</v>
+        <v>0.111604999999997</v>
       </c>
       <c r="K12" s="110"/>
       <c r="L12" s="136"/>
@@ -25938,11 +25965,11 @@
       </c>
       <c r="F13" s="134" t="n">
         <f aca="false">+E13+G13</f>
-        <v>7.599</v>
+        <v>7.535</v>
       </c>
       <c r="G13" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,110)/1000</f>
-        <v>0.099</v>
+        <v>0.035</v>
       </c>
       <c r="H13" s="109" t="n">
         <f aca="false">+(E13+E14)/2*D13</f>
@@ -25950,11 +25977,11 @@
       </c>
       <c r="I13" s="109" t="n">
         <f aca="false">+(F13+F14)/2*D13</f>
-        <v>129.76913</v>
+        <v>129.93234</v>
       </c>
       <c r="J13" s="109" t="n">
         <f aca="false">+I13-H13</f>
-        <v>0.919129999999996</v>
+        <v>1.08234000000002</v>
       </c>
       <c r="K13" s="110"/>
       <c r="L13" s="136"/>
@@ -25980,11 +26007,11 @@
       </c>
       <c r="F14" s="134" t="n">
         <f aca="false">+E14+G14</f>
-        <v>7.508</v>
+        <v>7.591</v>
       </c>
       <c r="G14" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,110)/1000</f>
-        <v>0.008</v>
+        <v>0.091</v>
       </c>
       <c r="H14" s="109" t="n">
         <f aca="false">+(E14+E15)/2*D14</f>
@@ -25992,11 +26019,11 @@
       </c>
       <c r="I14" s="109" t="n">
         <f aca="false">+(F14+F15)/2*D14</f>
-        <v>97.735435</v>
+        <v>98.396905</v>
       </c>
       <c r="J14" s="109" t="n">
         <f aca="false">+I14-H14</f>
-        <v>0.460435000000004</v>
+        <v>1.121905</v>
       </c>
       <c r="K14" s="110"/>
       <c r="L14" s="136"/>
@@ -26022,11 +26049,11 @@
       </c>
       <c r="F15" s="134" t="n">
         <f aca="false">+E15+G15</f>
-        <v>7.563</v>
+        <v>7.582</v>
       </c>
       <c r="G15" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,110)/1000</f>
-        <v>0.063</v>
+        <v>0.082</v>
       </c>
       <c r="H15" s="109" t="n">
         <f aca="false">+(E15+E16)/2*D15</f>
@@ -26034,11 +26061,11 @@
       </c>
       <c r="I15" s="109" t="n">
         <f aca="false">+(F15+F16)/2*D15</f>
-        <v>80.77818</v>
+        <v>80.80488</v>
       </c>
       <c r="J15" s="109" t="n">
         <f aca="false">+I15-H15</f>
-        <v>0.678179999999998</v>
+        <v>0.704880000000003</v>
       </c>
       <c r="K15" s="110"/>
       <c r="L15" s="136"/>
@@ -26064,11 +26091,11 @@
       </c>
       <c r="F16" s="134" t="n">
         <f aca="false">+E16+G16</f>
-        <v>7.564</v>
+        <v>7.55</v>
       </c>
       <c r="G16" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,110)/1000</f>
-        <v>0.064</v>
+        <v>0.05</v>
       </c>
       <c r="H16" s="109" t="n">
         <f aca="false">+(E16+E17)/2*D16</f>
@@ -26076,11 +26103,11 @@
       </c>
       <c r="I16" s="109" t="n">
         <f aca="false">+(F16+F17)/2*D16</f>
-        <v>129.676425</v>
+        <v>129.03255</v>
       </c>
       <c r="J16" s="109" t="n">
         <f aca="false">+I16-H16</f>
-        <v>0.901425000000018</v>
+        <v>0.257550000000009</v>
       </c>
       <c r="K16" s="110"/>
       <c r="L16" s="136"/>
@@ -26106,11 +26133,11 @@
       </c>
       <c r="F17" s="134" t="n">
         <f aca="false">+E17+G17</f>
-        <v>7.541</v>
+        <v>7.48</v>
       </c>
       <c r="G17" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,110)/1000</f>
-        <v>0.041</v>
+        <v>-0.02</v>
       </c>
       <c r="H17" s="109" t="n">
         <f aca="false">+(E17+E18)/2*D17</f>
@@ -26118,11 +26145,11 @@
       </c>
       <c r="I17" s="109" t="n">
         <f aca="false">+(F17+F18)/2*D17</f>
-        <v>129.04972</v>
+        <v>128.75783</v>
       </c>
       <c r="J17" s="109" t="n">
         <f aca="false">+I17-H17</f>
-        <v>0.274720000000002</v>
+        <v>-0.017169999999993</v>
       </c>
       <c r="K17" s="110"/>
       <c r="L17" s="136"/>
@@ -26148,11 +26175,11 @@
       </c>
       <c r="F18" s="134" t="n">
         <f aca="false">+E18+G18</f>
-        <v>7.491</v>
+        <v>7.518</v>
       </c>
       <c r="G18" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,110)/1000</f>
-        <v>-0.009</v>
+        <v>0.018</v>
       </c>
       <c r="H18" s="109" t="n">
         <f aca="false">+(E18+E19)/2*D18</f>
@@ -26160,11 +26187,11 @@
       </c>
       <c r="I18" s="109" t="n">
         <f aca="false">+(F18+F19)/2*D18</f>
-        <v>108.943065</v>
+        <v>109.232865</v>
       </c>
       <c r="J18" s="109" t="n">
         <f aca="false">+I18-H18</f>
-        <v>0.268064999999993</v>
+        <v>0.557865000000007</v>
       </c>
       <c r="K18" s="110"/>
       <c r="L18" s="136"/>
@@ -26187,11 +26214,11 @@
       </c>
       <c r="F19" s="134" t="n">
         <f aca="false">+E19+G19</f>
-        <v>7.546</v>
+        <v>7.559</v>
       </c>
       <c r="G19" s="67" t="n">
         <f aca="false">RANDBETWEEN(-30,110)/1000</f>
-        <v>0.046</v>
+        <v>0.059</v>
       </c>
       <c r="H19" s="109"/>
       <c r="I19" s="109"/>
@@ -26215,11 +26242,11 @@
       </c>
       <c r="I20" s="150" t="n">
         <f aca="false">SUM(I11:I19)</f>
-        <v>954.31554</v>
+        <v>952.12175</v>
       </c>
       <c r="J20" s="114" t="n">
         <f aca="false">+I20-H20</f>
-        <v>5.86554000000012</v>
+        <v>3.67175000000009</v>
       </c>
       <c r="K20" s="115"/>
       <c r="M20" s="117"/>

</xml_diff>